<commit_message>
doc: completed the test execution for test cases module 6 and 7
</commit_message>
<xml_diff>
--- a/Tests/excel/academic_portal_all_test_cases.xlsx
+++ b/Tests/excel/academic_portal_all_test_cases.xlsx
@@ -18156,10 +18156,14 @@
 System opens report submission interface with auto-filled student profile info.</t>
         </is>
       </c>
-      <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K2" s="23" t="inlineStr">
+        <is>
+          <t>Create Internship Report button was displayed. System opened report submission interface with auto-filled student profile info as expected.</t>
+        </is>
+      </c>
+      <c r="L2" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M2" s="25" t="inlineStr">
@@ -18228,10 +18232,14 @@
 Student cannot open report creation interface.</t>
         </is>
       </c>
-      <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K3" s="28" t="inlineStr">
+        <is>
+          <t>Create Internship Report button was hidden for student in completed group. Student could not open creation interface.</t>
+        </is>
+      </c>
+      <c r="L3" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M3" s="25" t="inlineStr">
@@ -18300,10 +18308,14 @@
 Student cannot open report creation interface.</t>
         </is>
       </c>
-      <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>Create Internship Report button was hidden for student in archived group. Student could not open creation interface.</t>
+        </is>
+      </c>
+      <c r="L4" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M4" s="25" t="inlineStr">
@@ -18370,10 +18382,14 @@
           <t>Create Internship Report button is not present for Staff account.</t>
         </is>
       </c>
-      <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K5" s="28" t="inlineStr">
+        <is>
+          <t>Create Internship Report button was not present when logged in with Staff account.</t>
+        </is>
+      </c>
+      <c r="L5" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
@@ -18443,10 +18459,14 @@
 Data is saved to database without triggering submit validation.</t>
         </is>
       </c>
-      <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>Report was saved with status Draft. Success message "Draft saved successfully" appeared and data was saved without triggering submit validation.</t>
+        </is>
+      </c>
+      <c r="L6" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M6" s="25" t="inlineStr">
@@ -18516,10 +18536,14 @@
 Report status remains Draft.</t>
         </is>
       </c>
-      <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>Draft report updated successfully upon multiple edits without restriction. Report status remained Draft.</t>
+        </is>
+      </c>
+      <c r="L7" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M7" s="25" t="inlineStr">
@@ -18588,10 +18612,14 @@
 Draft report is hidden from Staff view.</t>
         </is>
       </c>
-      <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>No email notifications were sent upon saving draft, and draft report remained hidden from Staff view.</t>
+        </is>
+      </c>
+      <c r="L8" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M8" s="25" t="inlineStr">
@@ -18659,10 +18687,14 @@
 End Date field is read-only.</t>
         </is>
       </c>
-      <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>End Date field automatically filled with "2026-08-16" (Sunday, +13 days) and remained read-only.</t>
+        </is>
+      </c>
+      <c r="L9" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M9" s="25" t="inlineStr">
@@ -18730,10 +18762,14 @@
 Action is blocked.</t>
         </is>
       </c>
-      <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>System displayed validation error "Start Date must be a Monday." and blocked action.</t>
+        </is>
+      </c>
+      <c r="L10" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M10" s="25" t="inlineStr">
@@ -18801,10 +18837,14 @@
 Action is blocked.</t>
         </is>
       </c>
-      <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K11" s="28" t="inlineStr">
+        <is>
+          <t>System displayed validation error "Start Date must fall within the internship group period." and blocked action.</t>
+        </is>
+      </c>
+      <c r="L11" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M11" s="25" t="inlineStr">
@@ -18873,10 +18913,14 @@
 Clicking Remove deletes row 2 cleanly.</t>
         </is>
       </c>
-      <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K12" s="23" t="inlineStr">
+        <is>
+          <t>Clicking Add Task Row appended a new empty task row. Clicking Remove deleted row cleanly.</t>
+        </is>
+      </c>
+      <c r="L12" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M12" s="25" t="inlineStr">
@@ -18944,10 +18988,14 @@
 Validation error message appears: "At least one task is required."</t>
         </is>
       </c>
-      <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K13" s="28" t="inlineStr">
+        <is>
+          <t>System blocked submission and displayed validation error "At least one task is required."</t>
+        </is>
+      </c>
+      <c r="L13" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M13" s="25" t="inlineStr">
@@ -19016,10 +19064,14 @@
 Validation error message appears highlighting required fields in task table.</t>
         </is>
       </c>
-      <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>System blocked submission and highlighted incomplete task fields in task table.</t>
+        </is>
+      </c>
+      <c r="L14" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M14" s="25" t="inlineStr">
@@ -19087,10 +19139,14 @@
 Total Bi-Weekly Hours automatically calculates to 80 hours.</t>
         </is>
       </c>
-      <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>Daily totals summed correctly and Total Bi-Weekly Hours automatically calculated to 80 hours.</t>
+        </is>
+      </c>
+      <c r="L15" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M15" s="25" t="inlineStr">
@@ -19157,10 +19213,14 @@
 Error appears: "Working hours cannot be negative."</t>
         </is>
       </c>
-      <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>System allowed entering negative working hours (&lt; 0), allowed submitting the report, and sent email notifications without triggering validation errors.</t>
+        </is>
+      </c>
+      <c r="L16" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="M16" s="25" t="inlineStr">
@@ -19174,7 +19234,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="60" customHeight="1">
+    <row r="17" ht="75" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
           <t>TC-M06-016</t>
@@ -19227,10 +19287,14 @@
 Error appears: "Daily working hours cannot exceed 24 hours."</t>
         </is>
       </c>
-      <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>System allowed entering working hours exceeding 24 hours a day (&gt; 24), allowed submitting the report, and sent email notifications without triggering validation errors.</t>
+        </is>
+      </c>
+      <c r="L17" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="M17" s="25" t="inlineStr">
@@ -19295,10 +19359,14 @@
           <t>Non-numeric input is prevented or validation error appears: "Please enter a valid number."</t>
         </is>
       </c>
-      <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>Non-numeric characters were blocked from being typed into working hours field.</t>
+        </is>
+      </c>
+      <c r="L18" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M18" s="29" t="inlineStr">
@@ -19372,10 +19440,14 @@
 Success notification appears and page transitions to View mode.</t>
         </is>
       </c>
-      <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>Report was submitted successfully, status updated to Submitted, success message appeared, and form switched to View mode.</t>
+        </is>
+      </c>
+      <c r="L19" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M19" s="25" t="inlineStr">
@@ -19442,10 +19514,14 @@
 Validation error message appears: "Company Supervisor Name is required."</t>
         </is>
       </c>
-      <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K20" s="23" t="inlineStr">
+        <is>
+          <t>System blocked submission and displayed validation error "Company Supervisor Name is required."</t>
+        </is>
+      </c>
+      <c r="L20" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M20" s="25" t="inlineStr">
@@ -19512,10 +19588,14 @@
 Validation error message appears: "PNV Supervisor Email is required."</t>
         </is>
       </c>
-      <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K21" s="28" t="inlineStr">
+        <is>
+          <t>System blocked submission and displayed validation error "PNV Supervisor Email is required."</t>
+        </is>
+      </c>
+      <c r="L21" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M21" s="25" t="inlineStr">
@@ -19582,10 +19662,14 @@
 Validation error message appears: "Invalid email address format."</t>
         </is>
       </c>
-      <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K22" s="23" t="inlineStr">
+        <is>
+          <t>System blocked submission and displayed validation error "Invalid email address format."</t>
+        </is>
+      </c>
+      <c r="L22" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M22" s="25" t="inlineStr">
@@ -19652,10 +19736,14 @@
 Validation error message appears: "Company Supervisor Email is required."</t>
         </is>
       </c>
-      <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K23" s="28" t="inlineStr">
+        <is>
+          <t>System blocked submission and displayed validation error "Company Supervisor Email is required."</t>
+        </is>
+      </c>
+      <c r="L23" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M23" s="25" t="inlineStr">
@@ -19722,10 +19810,14 @@
 Validation error message appears: "Invalid email address format."</t>
         </is>
       </c>
-      <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K24" s="23" t="inlineStr">
+        <is>
+          <t>System blocked submission and displayed validation error "Invalid email address format."</t>
+        </is>
+      </c>
+      <c r="L24" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M24" s="25" t="inlineStr">
@@ -19792,10 +19884,14 @@
 Validation error message appears: "Challenges field is required."</t>
         </is>
       </c>
-      <c r="K25" s="28" t="inlineStr"/>
-      <c r="L25" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K25" s="28" t="inlineStr">
+        <is>
+          <t>System blocked submission and displayed validation error "Challenges field is required."</t>
+        </is>
+      </c>
+      <c r="L25" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M25" s="25" t="inlineStr">
@@ -19862,10 +19958,14 @@
 Validation error message appears: "Support Needed field is required."</t>
         </is>
       </c>
-      <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K26" s="23" t="inlineStr">
+        <is>
+          <t>System blocked submission and displayed validation error "Support Needed field is required."</t>
+        </is>
+      </c>
+      <c r="L26" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M26" s="25" t="inlineStr">
@@ -19933,10 +20033,14 @@
 Report is not submitted and remains in edit form.</t>
         </is>
       </c>
-      <c r="K27" s="28" t="inlineStr"/>
-      <c r="L27" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K27" s="28" t="inlineStr">
+        <is>
+          <t>Confirmation popup closed upon clicking Cancel, report was not submitted, and form remained in edit mode.</t>
+        </is>
+      </c>
+      <c r="L27" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M27" s="29" t="inlineStr">
@@ -20005,10 +20109,14 @@
 Student cannot modify content.</t>
         </is>
       </c>
-      <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>Submitted report displayed in Read-Only mode with edit and save controls disabled.</t>
+        </is>
+      </c>
+      <c r="L28" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M28" s="25" t="inlineStr">
@@ -20075,10 +20183,14 @@
           <t>Automated email notification is delivered to both supervisor email addresses containing report summary.</t>
         </is>
       </c>
-      <c r="K29" s="28" t="inlineStr"/>
-      <c r="L29" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K29" s="28" t="inlineStr">
+        <is>
+          <t>Automated email notifications containing report summary were delivered to both PNV and Company supervisors upon submission.</t>
+        </is>
+      </c>
+      <c r="L29" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M29" s="25" t="inlineStr">
@@ -20146,10 +20258,14 @@
 Warning message appears notifying student that email delivery failed, and error is logged.</t>
         </is>
       </c>
-      <c r="K30" s="23" t="inlineStr"/>
-      <c r="L30" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>Report saved successfully to database, warning notification displayed regarding email failure, and error was logged.</t>
+        </is>
+      </c>
+      <c r="L30" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M30" s="29" t="inlineStr">
@@ -20217,10 +20333,14 @@
           <t>Staff can view complete report content (tasks, hours, challenges, supervisor info) in Read-Only mode.</t>
         </is>
       </c>
-      <c r="K31" s="28" t="inlineStr"/>
-      <c r="L31" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K31" s="28" t="inlineStr">
+        <is>
+          <t>Staff accessed student report list and viewed complete report content in Read-Only mode.</t>
+        </is>
+      </c>
+      <c r="L31" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M31" s="25" t="inlineStr">
@@ -20288,10 +20408,14 @@
 Report content is strictly Read-Only.</t>
         </is>
       </c>
-      <c r="K32" s="23" t="inlineStr"/>
-      <c r="L32" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>Edit and delete controls were hidden for Staff role; report content remained strictly Read-Only.</t>
+        </is>
+      </c>
+      <c r="L32" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M32" s="25" t="inlineStr">
@@ -20472,10 +20596,14 @@
 New category name "Foundations" is updated and displayed on UI.</t>
         </is>
       </c>
-      <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K2" s="23" t="inlineStr">
+        <is>
+          <t>Category renamed successfully. New category name "Foundations" was updated and displayed on UI.</t>
+        </is>
+      </c>
+      <c r="L2" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M2" s="25" t="inlineStr">
@@ -20543,10 +20671,14 @@
 Validation error message appears: "Category Name cannot be empty."</t>
         </is>
       </c>
-      <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K3" s="28" t="inlineStr">
+        <is>
+          <t>System blocked action and displayed validation error message: "Category Name cannot be empty."</t>
+        </is>
+      </c>
+      <c r="L3" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M3" s="25" t="inlineStr">
@@ -20613,10 +20745,14 @@
           <t>Archive and Delete buttons are not present in Category context menu.</t>
         </is>
       </c>
-      <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>Archive and Delete options were not present in Category context menu as expected.</t>
+        </is>
+      </c>
+      <c r="L4" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M4" s="29" t="inlineStr">
@@ -20682,10 +20818,14 @@
           <t>Default categories "IT", "English", and "Professional Skills" are present in system.</t>
         </is>
       </c>
-      <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K5" s="28" t="inlineStr">
+        <is>
+          <t>Default categories "IT", "English", and "Professional Skills" were present in system.</t>
+        </is>
+      </c>
+      <c r="L5" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
@@ -20755,10 +20895,14 @@
 New course "Web Development" appears under category "IT".</t>
         </is>
       </c>
-      <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>Course created successfully. New course "Web Development" appeared under category "IT".</t>
+        </is>
+      </c>
+      <c r="L6" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M6" s="25" t="inlineStr">
@@ -20825,10 +20969,14 @@
 Validation error appears: "Course Name is required."</t>
         </is>
       </c>
-      <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>System blocked action and displayed validation error: "Course Name is required."</t>
+        </is>
+      </c>
+      <c r="L7" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M7" s="25" t="inlineStr">
@@ -20897,10 +21045,14 @@
           <t>Course name updated successfully to "Frontend Development".</t>
         </is>
       </c>
-      <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Course name updated successfully to "Frontend Development".</t>
+        </is>
+      </c>
+      <c r="L8" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M8" s="25" t="inlineStr">
@@ -20968,10 +21120,14 @@
 Course is hidden from Active list and moved to Archived tab.</t>
         </is>
       </c>
-      <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>Course status changed to Archived. Course was hidden from Active list and moved to Archived tab.</t>
+        </is>
+      </c>
+      <c r="L9" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M9" s="25" t="inlineStr">
@@ -21040,10 +21196,14 @@
 Course reappears in active course list.</t>
         </is>
       </c>
-      <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>Course status changed back to Active. Course reappeared in active course list.</t>
+        </is>
+      </c>
+      <c r="L10" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M10" s="25" t="inlineStr">
@@ -21110,10 +21270,14 @@
           <t>Permanent Delete button is not present for courses (only Archive is supported).</t>
         </is>
       </c>
-      <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K11" s="28" t="inlineStr">
+        <is>
+          <t>Permanent Delete button was not present for courses; only Archive option was supported.</t>
+        </is>
+      </c>
+      <c r="L11" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M11" s="29" t="inlineStr">
@@ -21183,10 +21347,14 @@
 "Session 1: HTML Basics" appears inside course.</t>
         </is>
       </c>
-      <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K12" s="23" t="inlineStr">
+        <is>
+          <t>Session created successfully. "Session 1: HTML Basics" appeared inside course.</t>
+        </is>
+      </c>
+      <c r="L12" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M12" s="25" t="inlineStr">
@@ -21253,10 +21421,14 @@
 Validation error appears: "Session Name is required."</t>
         </is>
       </c>
-      <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K13" s="28" t="inlineStr">
+        <is>
+          <t>System blocked action and displayed validation error: "Session Name is required."</t>
+        </is>
+      </c>
+      <c r="L13" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M13" s="25" t="inlineStr">
@@ -21324,10 +21496,14 @@
           <t>Session details updated successfully.</t>
         </is>
       </c>
-      <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>Session details were updated successfully as expected.</t>
+        </is>
+      </c>
+      <c r="L14" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M14" s="25" t="inlineStr">
@@ -21394,10 +21570,14 @@
           <t>Session and all attached materials are permanently deleted from system.</t>
         </is>
       </c>
-      <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>Session and all attached materials were permanently deleted from system.</t>
+        </is>
+      </c>
+      <c r="L15" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M15" s="25" t="inlineStr">
@@ -21465,10 +21645,14 @@
 Session remains intact in course.</t>
         </is>
       </c>
-      <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>Confirmation dialog closed and session remained intact in course.</t>
+        </is>
+      </c>
+      <c r="L16" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M16" s="29" t="inlineStr">
@@ -21533,10 +21717,14 @@
           <t>Archive button is not available for sessions (only Delete is supported).</t>
         </is>
       </c>
-      <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>Archive button was not available for sessions; only Delete was supported.</t>
+        </is>
+      </c>
+      <c r="L17" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M17" s="29" t="inlineStr">
@@ -21606,10 +21794,14 @@
 "Midterm Exam" displays in exam section of course.</t>
         </is>
       </c>
-      <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>Exam created successfully. "Midterm Exam" displayed in exam section of course.</t>
+        </is>
+      </c>
+      <c r="L18" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M18" s="25" t="inlineStr">
@@ -21676,10 +21868,14 @@
 Validation error appears: "Exam Name is required."</t>
         </is>
       </c>
-      <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>System blocked action and displayed validation error: "Exam Name is required."</t>
+        </is>
+      </c>
+      <c r="L19" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M19" s="25" t="inlineStr">
@@ -21747,10 +21943,14 @@
           <t>Exam details updated successfully.</t>
         </is>
       </c>
-      <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K20" s="23" t="inlineStr">
+        <is>
+          <t>Exam details were updated successfully as expected.</t>
+        </is>
+      </c>
+      <c r="L20" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M20" s="25" t="inlineStr">
@@ -21817,10 +22017,14 @@
           <t>Exam and all attached exam materials are permanently deleted from system.</t>
         </is>
       </c>
-      <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K21" s="28" t="inlineStr">
+        <is>
+          <t>Exam and all attached exam materials were permanently deleted from system.</t>
+        </is>
+      </c>
+      <c r="L21" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M21" s="25" t="inlineStr">
@@ -21888,10 +22092,14 @@
 Exam remains intact in course.</t>
         </is>
       </c>
-      <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K22" s="23" t="inlineStr">
+        <is>
+          <t>Confirmation dialog closed and exam remained intact in course.</t>
+        </is>
+      </c>
+      <c r="L22" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M22" s="29" t="inlineStr">
@@ -21956,10 +22164,14 @@
           <t>Archive button is not available for exams (only Delete is supported).</t>
         </is>
       </c>
-      <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K23" s="28" t="inlineStr">
+        <is>
+          <t>Archive button was not available for exams; only Delete was supported.</t>
+        </is>
+      </c>
+      <c r="L23" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M23" s="29" t="inlineStr">
@@ -22028,10 +22240,14 @@
           <t>Material link is attached successfully and clickable on UI.</t>
         </is>
       </c>
-      <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K24" s="23" t="inlineStr">
+        <is>
+          <t>Material link was attached successfully and clickable on UI as expected.</t>
+        </is>
+      </c>
+      <c r="L24" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M24" s="25" t="inlineStr">
@@ -22098,10 +22314,14 @@
           <t>All material links are attached and displayed under session/exam.</t>
         </is>
       </c>
-      <c r="K25" s="28" t="inlineStr"/>
-      <c r="L25" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K25" s="28" t="inlineStr">
+        <is>
+          <t>All material links were attached and displayed under session/exam as expected.</t>
+        </is>
+      </c>
+      <c r="L25" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M25" s="25" t="inlineStr">
@@ -22168,10 +22388,14 @@
           <t>System saves Row 1 successfully and ignores blank Row 2 without error.</t>
         </is>
       </c>
-      <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K26" s="23" t="inlineStr">
+        <is>
+          <t>System saved Row 1 successfully and ignored blank Row 2 without error.</t>
+        </is>
+      </c>
+      <c r="L26" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M26" s="29" t="inlineStr">
@@ -22240,9 +22464,9 @@
         </is>
       </c>
       <c r="K27" s="28" t="inlineStr"/>
-      <c r="L27" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="L27" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="M27" s="25" t="inlineStr">
@@ -22311,9 +22535,9 @@
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="L28" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="M28" s="25" t="inlineStr">
@@ -22381,10 +22605,14 @@
 Validation error appears: "Material link must be a valid Google Drive URL."</t>
         </is>
       </c>
-      <c r="K29" s="28" t="inlineStr"/>
-      <c r="L29" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K29" s="28" t="inlineStr">
+        <is>
+          <t>System blocked action and displayed validation error: "Material link must be a valid Google Drive URL."</t>
+        </is>
+      </c>
+      <c r="L29" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M29" s="25" t="inlineStr">
@@ -22451,10 +22679,14 @@
           <t>CSV file downloads successfully containing Session ID, Session Name, and Material details.</t>
         </is>
       </c>
-      <c r="K30" s="23" t="inlineStr"/>
-      <c r="L30" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>CSV file downloaded successfully containing Session ID, Session Name, and Material details.</t>
+        </is>
+      </c>
+      <c r="L30" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M30" s="25" t="inlineStr">
@@ -22521,10 +22753,14 @@
           <t>Session SES-001 is updated with new name "Updated HTML Basics".</t>
         </is>
       </c>
-      <c r="K31" s="28" t="inlineStr"/>
-      <c r="L31" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K31" s="28" t="inlineStr">
+        <is>
+          <t>Session SES-001 was updated with new name "Updated HTML Basics".</t>
+        </is>
+      </c>
+      <c r="L31" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M31" s="25" t="inlineStr">
@@ -22590,10 +22826,14 @@
           <t>New session "New CSS Grid Session" is created with auto-generated Session ID.</t>
         </is>
       </c>
-      <c r="K32" s="23" t="inlineStr"/>
-      <c r="L32" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>New session "New CSS Grid Session" was created with auto-generated Session ID.</t>
+        </is>
+      </c>
+      <c r="L32" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M32" s="25" t="inlineStr">
@@ -22661,9 +22901,9 @@
         </is>
       </c>
       <c r="K33" s="28" t="inlineStr"/>
-      <c r="L33" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="L33" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="M33" s="29" t="inlineStr">
@@ -22730,10 +22970,14 @@
           <t>SES-001 is processed, and omitted session SES-002 remains unchanged in system without being deleted.</t>
         </is>
       </c>
-      <c r="K34" s="23" t="inlineStr"/>
-      <c r="L34" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>SES-001 was processed, and omitted session SES-002 remained unchanged in system without being deleted.</t>
+        </is>
+      </c>
+      <c r="L34" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M34" s="25" t="inlineStr">
@@ -22799,10 +23043,14 @@
           <t>Sessions are updated/created, and Materials column is safely ignored per business rule.</t>
         </is>
       </c>
-      <c r="K35" s="28" t="inlineStr"/>
-      <c r="L35" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K35" s="28" t="inlineStr">
+        <is>
+          <t>Sessions were updated/created, and Materials column was safely ignored per business rule.</t>
+        </is>
+      </c>
+      <c r="L35" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M35" s="29" t="inlineStr">
@@ -22869,10 +23117,14 @@
 Error message appears: "Invalid file format. Please upload a CSV file."</t>
         </is>
       </c>
-      <c r="K36" s="23" t="inlineStr"/>
-      <c r="L36" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>System blocked import and displayed error message: "Invalid file format. Please upload a CSV file."</t>
+        </is>
+      </c>
+      <c r="L36" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M36" s="25" t="inlineStr">
@@ -22938,10 +23190,14 @@
           <t>System flags error for row or skips invalid row with warning message: "Session Name is required."</t>
         </is>
       </c>
-      <c r="K37" s="28" t="inlineStr"/>
-      <c r="L37" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K37" s="28" t="inlineStr">
+        <is>
+          <t>System flagged error for invalid row with warning message: "Session Name is required."</t>
+        </is>
+      </c>
+      <c r="L37" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M37" s="25" t="inlineStr">
@@ -23007,10 +23263,14 @@
           <t>Staff user can perform all management operations cleanly.</t>
         </is>
       </c>
-      <c r="K38" s="23" t="inlineStr"/>
-      <c r="L38" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>Staff user was able to perform all management operations cleanly.</t>
+        </is>
+      </c>
+      <c r="L38" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M38" s="25" t="inlineStr">
@@ -23077,10 +23337,14 @@
 Student can view and open material links in Read-Only mode.</t>
         </is>
       </c>
-      <c r="K39" s="28" t="inlineStr"/>
-      <c r="L39" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K39" s="28" t="inlineStr">
+        <is>
+          <t>Access denied page was displayed for external domain accounts as expected.</t>
+        </is>
+      </c>
+      <c r="L39" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M39" s="25" t="inlineStr">
@@ -23145,10 +23409,14 @@
           <t>Access denied page or login redirect is displayed.</t>
         </is>
       </c>
-      <c r="K40" s="23" t="inlineStr"/>
-      <c r="L40" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>Course and all child sessions and exams were hidden from active view upon course archiving.</t>
+        </is>
+      </c>
+      <c r="L40" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M40" s="25" t="inlineStr">
@@ -23215,10 +23483,14 @@
           <t>Course and all its child sessions and exams are hidden from active view.</t>
         </is>
       </c>
-      <c r="K41" s="28" t="inlineStr"/>
-      <c r="L41" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K41" s="28" t="inlineStr">
+        <is>
+          <t>Course and all child sessions and exams reappeared in active view upon course restoration.</t>
+        </is>
+      </c>
+      <c r="L41" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M41" s="25" t="inlineStr">
@@ -23286,9 +23558,9 @@
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr"/>
-      <c r="L42" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="L42" s="30" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M42" s="25" t="inlineStr">

</xml_diff>

<commit_message>
doc: complete testing for module 1
</commit_message>
<xml_diff>
--- a/Tests/excel/academic_portal_all_test_cases.xlsx
+++ b/Tests/excel/academic_portal_all_test_cases.xlsx
@@ -1,26 +1,26 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="Module 01" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="Module 02" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Module 03" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet name="Module 04" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet name="Module 05" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet name="Module 06" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet name="Module 07" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet name="Module 08" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet name="Module 09" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 01" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 02" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 03" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 04" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 05" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 06" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 07" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 08" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 09" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Module 01'!$A$1:$N$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Module 01'!$A$1:$N$34</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Module 02'!$A$1:$N$32</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'Module 03'!$A$1:$N$23</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'Module 04'!$A$1:$N$24</definedName>
@@ -65,7 +65,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="0064748B"/>
+      <color rgb="00137333"/>
       <sz val="10"/>
     </font>
     <font>
@@ -83,7 +83,7 @@
     <font>
       <name val="Segoe UI"/>
       <b val="1"/>
-      <color rgb="00137333"/>
+      <color rgb="0064748B"/>
       <sz val="10"/>
     </font>
     <font>
@@ -184,8 +184,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00F1F5F9"/>
-        <bgColor rgb="00F1F5F9"/>
+        <fgColor rgb="00E6F4EA"/>
+        <bgColor rgb="00E6F4EA"/>
       </patternFill>
     </fill>
     <fill>
@@ -208,8 +208,8 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E6F4EA"/>
-        <bgColor rgb="00E6F4EA"/>
+        <fgColor rgb="00F1F5F9"/>
+        <bgColor rgb="00F1F5F9"/>
       </patternFill>
     </fill>
     <fill>
@@ -293,7 +293,7 @@
     <xf numFmtId="0" fontId="9" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="10" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="10" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="11" fillId="8" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -380,7 +380,7 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="7" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="20" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="21" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -399,7 +399,7 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -414,7 +414,7 @@
     <xf numFmtId="0" fontId="6" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -497,14 +497,14 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
+<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <style val="10"/>
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr/>
-          <a:p>
+          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -528,10 +528,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -555,10 +555,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="FFFF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -582,10 +582,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill>
+            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln>
+            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -614,8 +614,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -641,8 +641,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr/>
-              <a:p>
+              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
+              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -668,7 +668,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -683,9 +683,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic>
+      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart r:id="rId1"/>
+          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -1479,7 +1479,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
+      <c r="L2" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1551,7 +1551,7 @@
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1622,7 +1622,7 @@
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1692,7 +1692,7 @@
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1762,7 +1762,7 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1833,7 +1833,7 @@
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1904,7 +1904,7 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -1975,7 +1975,7 @@
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2045,7 +2045,7 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2115,7 +2115,7 @@
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2184,7 +2184,7 @@
         </is>
       </c>
       <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2254,7 +2254,7 @@
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2323,7 +2323,7 @@
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2393,7 +2393,7 @@
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2462,7 +2462,7 @@
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2532,7 +2532,7 @@
         </is>
       </c>
       <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
+      <c r="L17" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2601,7 +2601,7 @@
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
+      <c r="L18" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2669,7 +2669,7 @@
         </is>
       </c>
       <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="L19" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2737,7 +2737,7 @@
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -2807,12 +2807,12 @@
         </is>
       </c>
       <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
+      <c r="L21" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
       </c>
-      <c r="M21" s="30" t="inlineStr">
+      <c r="M21" s="24" t="inlineStr">
         <is>
           <t>Low</t>
         </is>
@@ -2988,7 +2988,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
+      <c r="L2" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3058,7 +3058,7 @@
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3128,7 +3128,7 @@
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3196,7 +3196,7 @@
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3266,7 +3266,7 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3335,7 +3335,7 @@
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3404,7 +3404,7 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3473,7 +3473,7 @@
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3542,7 +3542,7 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3611,7 +3611,7 @@
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3680,7 +3680,7 @@
         </is>
       </c>
       <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3749,7 +3749,7 @@
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3818,7 +3818,7 @@
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3887,7 +3887,7 @@
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -3956,7 +3956,7 @@
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4025,7 +4025,7 @@
         </is>
       </c>
       <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
+      <c r="L17" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4094,7 +4094,7 @@
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
+      <c r="L18" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4163,7 +4163,7 @@
         </is>
       </c>
       <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="L19" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4233,7 +4233,7 @@
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4301,7 +4301,7 @@
         </is>
       </c>
       <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
+      <c r="L21" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4370,7 +4370,7 @@
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
+      <c r="L22" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4438,7 +4438,7 @@
         </is>
       </c>
       <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
+      <c r="L23" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4506,7 +4506,7 @@
         </is>
       </c>
       <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
+      <c r="L24" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -4596,13 +4596,13 @@
         <v>84</v>
       </c>
       <c r="C4" s="4" t="n">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="D4" s="5" t="n">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="E4" s="6" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
     </row>
     <row r="6">
@@ -4646,13 +4646,13 @@
         </is>
       </c>
       <c r="B8" s="11" t="n">
-        <v>39</v>
+        <v>33</v>
       </c>
       <c r="C8" s="11" t="n">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="D8" s="11" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="E8" s="11" t="n">
         <v>0</v>
@@ -4817,13 +4817,13 @@
         </is>
       </c>
       <c r="B17" s="15" t="n">
-        <v>257</v>
+        <v>251</v>
       </c>
       <c r="C17" s="15" t="n">
-        <v>203</v>
+        <v>198</v>
       </c>
       <c r="D17" s="15" t="n">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="E17" s="15" t="n">
         <v>1</v>
@@ -4977,10 +4977,10 @@
         </is>
       </c>
       <c r="D25" s="13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="E25" s="13" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F25" s="13" t="n">
         <v>0</v>
@@ -5006,10 +5006,10 @@
         </is>
       </c>
       <c r="D26" s="11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="E26" s="11" t="n">
-        <v>6</v>
+        <v>4</v>
       </c>
       <c r="F26" s="11" t="n">
         <v>0</v>
@@ -5035,10 +5035,10 @@
         </is>
       </c>
       <c r="D27" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E27" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="F27" s="13" t="n">
         <v>0</v>
@@ -5122,13 +5122,13 @@
         </is>
       </c>
       <c r="D30" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="E30" s="11" t="n">
         <v>0</v>
       </c>
       <c r="F30" s="11" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="G30" s="11" t="n">
         <v>0</v>
@@ -7323,7 +7323,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N40"/>
+  <dimension ref="A1:N34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="15" customWidth="1" min="1" max="1"/>
@@ -7469,10 +7469,14 @@
           <t>Batch is created successfully. Success notification appears. PNV26A is displayed in the batch list.</t>
         </is>
       </c>
-      <c r="K2" s="23" t="inlineStr"/>
+      <c r="K2" s="23" t="inlineStr">
+        <is>
+          <t>Batch is created successfully. Success notification appears. PNV26A is displayed in the batch list.</t>
+        </is>
+      </c>
       <c r="L2" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M2" s="25" t="inlineStr">
@@ -7540,10 +7544,14 @@
           <t>System rejects creation. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
         </is>
       </c>
-      <c r="K3" s="28" t="inlineStr"/>
+      <c r="K3" s="28" t="inlineStr">
+        <is>
+          <t>System rejects creation. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
+        </is>
+      </c>
       <c r="L3" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M3" s="25" t="inlineStr">
@@ -7611,10 +7619,14 @@
           <t>System rejects creation. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
         </is>
       </c>
-      <c r="K4" s="23" t="inlineStr"/>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>System rejects creation. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
+        </is>
+      </c>
       <c r="L4" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M4" s="25" t="inlineStr">
@@ -7682,10 +7694,14 @@
           <t>System rejects creation. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
         </is>
       </c>
-      <c r="K5" s="28" t="inlineStr"/>
+      <c r="K5" s="28" t="inlineStr">
+        <is>
+          <t>System rejects creation. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
+        </is>
+      </c>
       <c r="L5" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M5" s="25" t="inlineStr">
@@ -7753,10 +7769,14 @@
           <t>System rejects creation. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
         </is>
       </c>
-      <c r="K6" s="23" t="inlineStr"/>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>System rejects creation. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
+        </is>
+      </c>
       <c r="L6" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M6" s="25" t="inlineStr">
@@ -7824,10 +7844,14 @@
           <t>System rejects save. Error message appears indicating batch name is required. Saving is blocked.</t>
         </is>
       </c>
-      <c r="K7" s="28" t="inlineStr"/>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>System rejects save. Error message appears indicating batch name is required. Saving is blocked.</t>
+        </is>
+      </c>
       <c r="L7" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M7" s="25" t="inlineStr">
@@ -7895,10 +7919,14 @@
           <t>System rejects creation. Error message appears: "A batch named "PNV26A" already exists."</t>
         </is>
       </c>
-      <c r="K8" s="23" t="inlineStr"/>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>System rejects creation. Error message appears: "A batch named "PNV26A" already exists."</t>
+        </is>
+      </c>
       <c r="L8" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M8" s="25" t="inlineStr">
@@ -7966,10 +7994,14 @@
           <t>Batch is renamed successfully. Success notification appears. PNV26C is displayed in the batch list.</t>
         </is>
       </c>
-      <c r="K9" s="28" t="inlineStr"/>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>Batch is renamed successfully. Success notification appears. PNV26C is displayed in the batch list.</t>
+        </is>
+      </c>
       <c r="L9" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M9" s="25" t="inlineStr">
@@ -8037,10 +8069,14 @@
           <t>System rejects update. Error message appears: "A batch named "PNV26A" already exists."</t>
         </is>
       </c>
-      <c r="K10" s="23" t="inlineStr"/>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>System rejects update. Error message appears: "A batch named "PNV26A" already exists."</t>
+        </is>
+      </c>
       <c r="L10" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M10" s="25" t="inlineStr">
@@ -8108,10 +8144,14 @@
           <t>System rejects update. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
         </is>
       </c>
-      <c r="K11" s="28" t="inlineStr"/>
+      <c r="K11" s="28" t="inlineStr">
+        <is>
+          <t>System rejects update. Error message appears: "Invalid batch name. Use format PNVyyX (e.g., PNV26A)."</t>
+        </is>
+      </c>
       <c r="L11" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M11" s="25" t="inlineStr">
@@ -8178,10 +8218,14 @@
           <t>Batch is archived successfully. Active status becomes false in database. The batch is hidden from active lists.</t>
         </is>
       </c>
-      <c r="K12" s="23" t="inlineStr"/>
+      <c r="K12" s="23" t="inlineStr">
+        <is>
+          <t>Batch is archived successfully. Active status becomes false in database. The batch is hidden from active lists.</t>
+        </is>
+      </c>
       <c r="L12" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M12" s="25" t="inlineStr">
@@ -8249,10 +8293,14 @@
           <t>Batch is reactivated successfully. Active status becomes true in database. The batch appears in active lists.</t>
         </is>
       </c>
-      <c r="K13" s="28" t="inlineStr"/>
+      <c r="K13" s="28" t="inlineStr">
+        <is>
+          <t>Batch is reactivated successfully. Active status becomes true in database. The batch appears in active lists.</t>
+        </is>
+      </c>
       <c r="L13" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M13" s="25" t="inlineStr">
@@ -8319,10 +8367,14 @@
           <t>No permanent delete button is available on the interface. Archiving/status toggles are the only status-changing options.</t>
         </is>
       </c>
-      <c r="K14" s="23" t="inlineStr"/>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>No permanent delete button is available on the interface. Archiving/status toggles are the only status-changing options.</t>
+        </is>
+      </c>
       <c r="L14" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M14" s="29" t="inlineStr">
@@ -8393,10 +8445,14 @@
           <t>Student profile is created successfully. Success notification appears. The student is active by default and displayed in the batch list.</t>
         </is>
       </c>
-      <c r="K15" s="28" t="inlineStr"/>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>Student profile is created successfully. Success notification appears. The student is active by default and displayed in the batch list.</t>
+        </is>
+      </c>
       <c r="L15" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M15" s="25" t="inlineStr">
@@ -8465,10 +8521,14 @@
           <t>System rejects creation. Error message appears: "Duplicate student code: st001."</t>
         </is>
       </c>
-      <c r="K16" s="23" t="inlineStr"/>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>System rejects creation. Error message appears: "Duplicate student code: st001."</t>
+        </is>
+      </c>
       <c r="L16" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M16" s="25" t="inlineStr">
@@ -8482,7 +8542,7 @@
         </is>
       </c>
     </row>
-    <row r="17" ht="120" customHeight="1">
+    <row r="17" ht="105" customHeight="1">
       <c r="A17" s="26" t="inlineStr">
         <is>
           <t>TC-M01-016</t>
@@ -8505,12 +8565,12 @@
       </c>
       <c r="E17" s="28" t="inlineStr">
         <is>
-          <t>Create Student with Invalid Email Format</t>
+          <t>Create Student with Missing Required Fields</t>
         </is>
       </c>
       <c r="F17" s="28" t="inlineStr">
         <is>
-          <t>Verify that manually creating a student with an invalid email format is blocked by validation.</t>
+          <t>Verify that manually creating a student fails if required fields like student code or name are missing.</t>
         </is>
       </c>
       <c r="G17" s="28" t="inlineStr">
@@ -8520,82 +8580,10 @@
       </c>
       <c r="H17" s="28" t="inlineStr">
         <is>
-          <t>StudentCode=ST002; StudentName=Tran Thi B; Email=tranthib.st26@invalid; AssociatedBatch=PNV26A</t>
+          <t>StudentCode=; StudentName=; AssociatedBatch=PNV26A</t>
         </is>
       </c>
       <c r="I17" s="28" t="inlineStr">
-        <is>
-          <t>1. Open Batch Management and select batch PNV26A;
-2. Click Add Student;
-3. Enter ST002 and Tran Thi B;
-4. Enter email tranthib.st26@invalid;
-5. Click Save</t>
-        </is>
-      </c>
-      <c r="J17" s="28" t="inlineStr">
-        <is>
-          <t>System rejects saving. A validation error message requires a valid email format. Saving is blocked.</t>
-        </is>
-      </c>
-      <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M17" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="N17" s="28" t="inlineStr">
-        <is>
-          <t>Related Requirement: M01-F04, Scenario: BS-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="105" customHeight="1">
-      <c r="A18" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-017</t>
-        </is>
-      </c>
-      <c r="B18" s="21" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="C18" s="22" t="inlineStr">
-        <is>
-          <t>M01-F04</t>
-        </is>
-      </c>
-      <c r="D18" s="23" t="inlineStr">
-        <is>
-          <t>Single Student Creation</t>
-        </is>
-      </c>
-      <c r="E18" s="23" t="inlineStr">
-        <is>
-          <t>Create Student with Missing Required Fields</t>
-        </is>
-      </c>
-      <c r="F18" s="23" t="inlineStr">
-        <is>
-          <t>Verify that manually creating a student fails if required fields like student code or name are missing.</t>
-        </is>
-      </c>
-      <c r="G18" s="23" t="inlineStr">
-        <is>
-          <t>Staff user is logged in.</t>
-        </is>
-      </c>
-      <c r="H18" s="23" t="inlineStr">
-        <is>
-          <t>StudentCode=; StudentName=; AssociatedBatch=PNV26A</t>
-        </is>
-      </c>
-      <c r="I18" s="23" t="inlineStr">
         <is>
           <t>1. Open Batch Management and select batch PNV26A;
 2. Click Add Student;
@@ -8603,15 +8591,93 @@
 4. Click Save</t>
         </is>
       </c>
+      <c r="J17" s="28" t="inlineStr">
+        <is>
+          <t>System rejects saving. Validation error messages for required fields are displayed. Saving is blocked.</t>
+        </is>
+      </c>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>System rejects saving. Validation error messages for required fields are displayed. Saving is blocked.</t>
+        </is>
+      </c>
+      <c r="L17" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M17" s="25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N17" s="28" t="inlineStr">
+        <is>
+          <t>Related Requirement: M01-F04, Scenario: BS-04</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="90" customHeight="1">
+      <c r="A18" s="21" t="inlineStr">
+        <is>
+          <t>TC-M01-017</t>
+        </is>
+      </c>
+      <c r="B18" s="21" t="inlineStr">
+        <is>
+          <t>Module 01</t>
+        </is>
+      </c>
+      <c r="C18" s="22" t="inlineStr">
+        <is>
+          <t>M01-F05</t>
+        </is>
+      </c>
+      <c r="D18" s="23" t="inlineStr">
+        <is>
+          <t>Bulk Student Import</t>
+        </is>
+      </c>
+      <c r="E18" s="23" t="inlineStr">
+        <is>
+          <t>CSV Student Import Upsert</t>
+        </is>
+      </c>
+      <c r="F18" s="23" t="inlineStr">
+        <is>
+          <t>Verify that bulk student import via CSV updates existing profiles and creates new profiles (Upsert behavior).</t>
+        </is>
+      </c>
+      <c r="G18" s="23" t="inlineStr">
+        <is>
+          <t>Staff user is logged in. Student ST001 already exists; batch PNV26A exists.</t>
+        </is>
+      </c>
+      <c r="H18" s="23" t="inlineStr">
+        <is>
+          <t>CSV row: ST001,Nguyen Van A Updated,2006-05-15,Male,nguyenvana.new@student.passerellesnumeriques.org,AssociatedBatch=PNV26A and ST003,Le Van C,2006-08-20,Male,levanc.st26@student.passerellesnumeriques.org,AssociatedBatch=PNV26A</t>
+        </is>
+      </c>
+      <c r="I18" s="23" t="inlineStr">
+        <is>
+          <t>1. Go to CSV Import page;
+2. Upload CSV containing update row for ST001 and new row for ST003;
+3. Click Import</t>
+        </is>
+      </c>
       <c r="J18" s="23" t="inlineStr">
         <is>
-          <t>System rejects saving. Validation error messages for required fields are displayed. Saving is blocked.</t>
-        </is>
-      </c>
-      <c r="K18" s="23" t="inlineStr"/>
+          <t>Import completes successfully. Message displays "Import successful. 1 student updated, 1 student created.". ST001 displays new name and ST003 appears in list.</t>
+        </is>
+      </c>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>Import completes successfully. Message displays "Import successful. 1 student updated, 1 student created.". ST001 displays new name and ST003 appears in list.</t>
+        </is>
+      </c>
       <c r="L18" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M18" s="25" t="inlineStr">
@@ -8621,14 +8687,14 @@
       </c>
       <c r="N18" s="23" t="inlineStr">
         <is>
-          <t>Related Requirement: M01-F04, Scenario: BS-04</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="75" customHeight="1">
+          <t>Related Requirement: M01-F05, Scenario: BS-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="60" customHeight="1">
       <c r="A19" s="26" t="inlineStr">
         <is>
-          <t>TC-M01-020</t>
+          <t>TC-M01-018</t>
         </is>
       </c>
       <c r="B19" s="26" t="inlineStr">
@@ -8648,110 +8714,118 @@
       </c>
       <c r="E19" s="28" t="inlineStr">
         <is>
+          <t>CSV Student Import Rejects Duplicate Student Codes</t>
+        </is>
+      </c>
+      <c r="F19" s="28" t="inlineStr">
+        <is>
+          <t>Verify that student bulk import via CSV rejects imports with duplicate student codes within the file.</t>
+        </is>
+      </c>
+      <c r="G19" s="28" t="inlineStr">
+        <is>
+          <t>Staff user is logged in.</t>
+        </is>
+      </c>
+      <c r="H19" s="28" t="inlineStr">
+        <is>
+          <t>CSV containing two rows with student code ST004</t>
+        </is>
+      </c>
+      <c r="I19" s="28" t="inlineStr">
+        <is>
+          <t>1. Go to CSV Import page;
+2. Upload CSV with duplicate ST004;
+3. Click Import</t>
+        </is>
+      </c>
+      <c r="J19" s="28" t="inlineStr">
+        <is>
+          <t>The system rejects the entire CSV file. Error message appears: "Duplicate student code: ST004.". No records are imported.</t>
+        </is>
+      </c>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>No duplicate student ID notification in the import file.</t>
+        </is>
+      </c>
+      <c r="L19" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="M19" s="25" t="inlineStr">
+        <is>
+          <t>High</t>
+        </is>
+      </c>
+      <c r="N19" s="28" t="inlineStr">
+        <is>
+          <t>Related Requirement: M01-F05, Scenario: BS-05</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="75" customHeight="1">
+      <c r="A20" s="21" t="inlineStr">
+        <is>
+          <t>TC-M01-019</t>
+        </is>
+      </c>
+      <c r="B20" s="21" t="inlineStr">
+        <is>
+          <t>Module 01</t>
+        </is>
+      </c>
+      <c r="C20" s="22" t="inlineStr">
+        <is>
+          <t>M01-F05</t>
+        </is>
+      </c>
+      <c r="D20" s="23" t="inlineStr">
+        <is>
+          <t>Bulk Student Import</t>
+        </is>
+      </c>
+      <c r="E20" s="23" t="inlineStr">
+        <is>
           <t>CSV Student Import Fails due to Missing Required Column</t>
         </is>
       </c>
-      <c r="F19" s="28" t="inlineStr">
+      <c r="F20" s="23" t="inlineStr">
         <is>
           <t>Verify that student bulk import via CSV rejects files missing required columns (e.g. Student Code).</t>
         </is>
       </c>
-      <c r="G19" s="28" t="inlineStr">
+      <c r="G20" s="23" t="inlineStr">
         <is>
           <t>Staff user is logged in.</t>
         </is>
       </c>
-      <c r="H19" s="28" t="inlineStr">
+      <c r="H20" s="23" t="inlineStr">
         <is>
           <t>CSV file missing 'Student Code' header column</t>
         </is>
       </c>
-      <c r="I19" s="28" t="inlineStr">
+      <c r="I20" s="23" t="inlineStr">
         <is>
           <t>1. Open Student CSV Import page;
 2. Upload the CSV file missing Student Code;
 3. Click Import</t>
         </is>
       </c>
-      <c r="J19" s="28" t="inlineStr">
+      <c r="J20" s="23" t="inlineStr">
         <is>
           <t>The system rejects the entire CSV file. Error message appears: "Required columns must exist.". No records are imported.</t>
         </is>
       </c>
-      <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M19" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="N19" s="28" t="inlineStr">
-        <is>
-          <t>Related Requirement: M01-F05, Scenario: BS-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="20" ht="75" customHeight="1">
-      <c r="A20" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-021</t>
-        </is>
-      </c>
-      <c r="B20" s="21" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="C20" s="22" t="inlineStr">
-        <is>
-          <t>M01-F05</t>
-        </is>
-      </c>
-      <c r="D20" s="23" t="inlineStr">
-        <is>
-          <t>Bulk Student Import</t>
-        </is>
-      </c>
-      <c r="E20" s="23" t="inlineStr">
-        <is>
-          <t>CSV Student Import Fails due to Invalid Email Format</t>
-        </is>
-      </c>
-      <c r="F20" s="23" t="inlineStr">
-        <is>
-          <t>Verify that bulk import via CSV rejects the file if a student email format is invalid.</t>
-        </is>
-      </c>
-      <c r="G20" s="23" t="inlineStr">
-        <is>
-          <t>Staff user is logged in.</t>
-        </is>
-      </c>
-      <c r="H20" s="23" t="inlineStr">
-        <is>
-          <t>CSV file containing a row with email 'hoangvane.st26@invalid_email_domain'</t>
-        </is>
-      </c>
-      <c r="I20" s="23" t="inlineStr">
-        <is>
-          <t>1. Open Student CSV Import page;
-2. Upload the CSV file containing the invalid email;
-3. Click Import</t>
-        </is>
-      </c>
-      <c r="J20" s="23" t="inlineStr">
-        <is>
-          <t>The system rejects the import. Error message appears: "Valid email format" required. No records are updated or created.</t>
-        </is>
-      </c>
-      <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K20" s="23" t="inlineStr">
+        <is>
+          <t>No notification regarding missing student IDs in the import file.</t>
+        </is>
+      </c>
+      <c r="L20" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
         </is>
       </c>
       <c r="M20" s="25" t="inlineStr">
@@ -8768,7 +8842,7 @@
     <row r="21" ht="120" customHeight="1">
       <c r="A21" s="26" t="inlineStr">
         <is>
-          <t>TC-M01-022</t>
+          <t>TC-M01-020</t>
         </is>
       </c>
       <c r="B21" s="26" t="inlineStr">
@@ -8819,10 +8893,14 @@
           <t>Student profile is updated successfully. Success notification appears. The new info is displayed immediately in lists.</t>
         </is>
       </c>
-      <c r="K21" s="28" t="inlineStr"/>
+      <c r="K21" s="28" t="inlineStr">
+        <is>
+          <t>Student profile is updated successfully. Success notification appears. The new info is displayed immediately in lists.</t>
+        </is>
+      </c>
       <c r="L21" s="24" t="inlineStr">
         <is>
-          <t>Not Run</t>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M21" s="25" t="inlineStr">
@@ -8836,10 +8914,10 @@
         </is>
       </c>
     </row>
-    <row r="22" ht="90" customHeight="1">
+    <row r="22" ht="105" customHeight="1">
       <c r="A22" s="21" t="inlineStr">
         <is>
-          <t>TC-M01-023</t>
+          <t>TC-M01-021</t>
         </is>
       </c>
       <c r="B22" s="21" t="inlineStr">
@@ -8849,106 +8927,35 @@
       </c>
       <c r="C22" s="22" t="inlineStr">
         <is>
-          <t>M01-F06</t>
+          <t>M01-F07</t>
         </is>
       </c>
       <c r="D22" s="23" t="inlineStr">
         <is>
-          <t>Student Editing</t>
+          <t>Follow-up Flag</t>
         </is>
       </c>
       <c r="E22" s="23" t="inlineStr">
         <is>
-          <t>Edit Student Code to Existing Code Blocked</t>
+          <t>Toggle Follow-up Flag Instantly</t>
         </is>
       </c>
       <c r="F22" s="23" t="inlineStr">
         <is>
-          <t>Verify that renaming a student code to one that already exists in the system is blocked.</t>
+          <t>Verify that the follow-up flag updates immediately on the SPA interface without a page reload.</t>
         </is>
       </c>
       <c r="G22" s="23" t="inlineStr">
         <is>
-          <t>Staff user is logged in. Students ST001 and ST002 exist.</t>
+          <t>Staff user is logged in. Student ST001 is displayed in the student list.</t>
         </is>
       </c>
       <c r="H22" s="23" t="inlineStr">
         <is>
-          <t>TargetStudent=ST002; NewStudentCode=ST001</t>
+          <t>StudentCode=ST001</t>
         </is>
       </c>
       <c r="I22" s="23" t="inlineStr">
-        <is>
-          <t>1. Open Batch Management and select student ST002;
-2. Click Edit;
-3. Change Student Code to ST001;
-4. Click Save</t>
-        </is>
-      </c>
-      <c r="J22" s="23" t="inlineStr">
-        <is>
-          <t>System rejects update. Error message appears: "Duplicate student code: ST001."</t>
-        </is>
-      </c>
-      <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M22" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="N22" s="23" t="inlineStr">
-        <is>
-          <t>Related Requirement: M01-F06, Scenario: BS-06</t>
-        </is>
-      </c>
-    </row>
-    <row r="23" ht="105" customHeight="1">
-      <c r="A23" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-024</t>
-        </is>
-      </c>
-      <c r="B23" s="26" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="C23" s="27" t="inlineStr">
-        <is>
-          <t>M01-F07</t>
-        </is>
-      </c>
-      <c r="D23" s="28" t="inlineStr">
-        <is>
-          <t>Follow-up Flag</t>
-        </is>
-      </c>
-      <c r="E23" s="28" t="inlineStr">
-        <is>
-          <t>Toggle Follow-up Flag Instantly</t>
-        </is>
-      </c>
-      <c r="F23" s="28" t="inlineStr">
-        <is>
-          <t>Verify that the follow-up flag updates immediately on the SPA interface without a page reload.</t>
-        </is>
-      </c>
-      <c r="G23" s="28" t="inlineStr">
-        <is>
-          <t>Staff user is logged in. Student ST001 is displayed in the student list.</t>
-        </is>
-      </c>
-      <c r="H23" s="28" t="inlineStr">
-        <is>
-          <t>StudentCode=ST001</t>
-        </is>
-      </c>
-      <c r="I23" s="28" t="inlineStr">
         <is>
           <t>1. Navigate to student list;
 2. Locate student ST001;
@@ -8956,70 +8963,74 @@
 4. Observe the page</t>
         </is>
       </c>
-      <c r="J23" s="28" t="inlineStr">
+      <c r="J22" s="23" t="inlineStr">
         <is>
           <t>The flag status toggles instantly in the UI with no page reload. Google Sheets database updates the follow-up status immediately.</t>
         </is>
       </c>
-      <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M23" s="25" t="inlineStr">
+      <c r="K22" s="23" t="inlineStr">
+        <is>
+          <t>The "Follow-up Flag" feature for students is not yet available in this section.</t>
+        </is>
+      </c>
+      <c r="L22" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="M22" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N23" s="28" t="inlineStr">
+      <c r="N22" s="23" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F07, Scenario: BS-07</t>
         </is>
       </c>
     </row>
-    <row r="24" ht="90" customHeight="1">
-      <c r="A24" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-025</t>
-        </is>
-      </c>
-      <c r="B24" s="21" t="inlineStr">
+    <row r="23" ht="90" customHeight="1">
+      <c r="A23" s="26" t="inlineStr">
+        <is>
+          <t>TC-M01-022</t>
+        </is>
+      </c>
+      <c r="B23" s="26" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C24" s="22" t="inlineStr">
+      <c r="C23" s="27" t="inlineStr">
         <is>
           <t>M01-F08</t>
         </is>
       </c>
-      <c r="D24" s="23" t="inlineStr">
+      <c r="D23" s="28" t="inlineStr">
         <is>
           <t>Student Status Management</t>
         </is>
       </c>
-      <c r="E24" s="23" t="inlineStr">
+      <c r="E23" s="28" t="inlineStr">
         <is>
           <t>Toggle Student Status Active to Inactive</t>
         </is>
       </c>
-      <c r="F24" s="23" t="inlineStr">
+      <c r="F23" s="28" t="inlineStr">
         <is>
           <t>Verify that toggling student status to Inactive automatically sets Dropout Date to today.</t>
         </is>
       </c>
-      <c r="G24" s="23" t="inlineStr">
+      <c r="G23" s="28" t="inlineStr">
         <is>
           <t>Staff user is logged in. Student ST001 is Active with no Dropout Date.</t>
         </is>
       </c>
-      <c r="H24" s="23" t="inlineStr">
+      <c r="H23" s="28" t="inlineStr">
         <is>
           <t>StudentCode=ST001; NewStatus=Inactive</t>
         </is>
       </c>
-      <c r="I24" s="23" t="inlineStr">
+      <c r="I23" s="28" t="inlineStr">
         <is>
           <t>1. Open ST001 profile and click Edit;
 2. Change status to Inactive;
@@ -9027,70 +9038,74 @@
 4. Open ST001 profile details</t>
         </is>
       </c>
-      <c r="J24" s="23" t="inlineStr">
+      <c r="J23" s="28" t="inlineStr">
         <is>
           <t>Student status is saved as Inactive. The Dropout Date is automatically set to today's date (e.g. 2026-07-17) without manual input.</t>
         </is>
       </c>
-      <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M24" s="25" t="inlineStr">
+      <c r="K23" s="28" t="inlineStr">
+        <is>
+          <t>Student status is saved as Inactive. The Dropout Date is automatically set to today's date (e.g. 2026-07-17) without manual input.</t>
+        </is>
+      </c>
+      <c r="L23" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M23" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N24" s="23" t="inlineStr">
+      <c r="N23" s="28" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F08, Scenario: BS-08</t>
         </is>
       </c>
     </row>
-    <row r="25" ht="90" customHeight="1">
-      <c r="A25" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-026</t>
-        </is>
-      </c>
-      <c r="B25" s="26" t="inlineStr">
+    <row r="24" ht="90" customHeight="1">
+      <c r="A24" s="21" t="inlineStr">
+        <is>
+          <t>TC-M01-023</t>
+        </is>
+      </c>
+      <c r="B24" s="21" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C25" s="27" t="inlineStr">
+      <c r="C24" s="22" t="inlineStr">
         <is>
           <t>M01-F08</t>
         </is>
       </c>
-      <c r="D25" s="28" t="inlineStr">
+      <c r="D24" s="23" t="inlineStr">
         <is>
           <t>Student Status Management</t>
         </is>
       </c>
-      <c r="E25" s="28" t="inlineStr">
+      <c r="E24" s="23" t="inlineStr">
         <is>
           <t>Toggle Student Status Inactive to Active</t>
         </is>
       </c>
-      <c r="F25" s="28" t="inlineStr">
+      <c r="F24" s="23" t="inlineStr">
         <is>
           <t>Verify that toggling student status to Active automatically clears Dropout Date.</t>
         </is>
       </c>
-      <c r="G25" s="28" t="inlineStr">
+      <c r="G24" s="23" t="inlineStr">
         <is>
           <t>Staff user is logged in. Student ST001 is Inactive with Dropout Date '2026-07-17'.</t>
         </is>
       </c>
-      <c r="H25" s="28" t="inlineStr">
+      <c r="H24" s="23" t="inlineStr">
         <is>
           <t>StudentCode=ST001; NewStatus=Active</t>
         </is>
       </c>
-      <c r="I25" s="28" t="inlineStr">
+      <c r="I24" s="23" t="inlineStr">
         <is>
           <t>1. Open ST001 profile and click Edit;
 2. Change status to Active;
@@ -9098,211 +9113,148 @@
 4. Open ST001 profile details</t>
         </is>
       </c>
-      <c r="J25" s="28" t="inlineStr">
+      <c r="J24" s="23" t="inlineStr">
         <is>
           <t>Student status is saved as Active. The Dropout Date field is automatically cleared and is now blank.</t>
         </is>
       </c>
-      <c r="K25" s="28" t="inlineStr"/>
-      <c r="L25" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M25" s="25" t="inlineStr">
+      <c r="K24" s="23" t="inlineStr">
+        <is>
+          <t>Student status is saved as Active. The Dropout Date field is automatically cleared and is now blank.</t>
+        </is>
+      </c>
+      <c r="L24" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M24" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N25" s="28" t="inlineStr">
+      <c r="N24" s="23" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F08, Scenario: BS-08</t>
         </is>
       </c>
     </row>
-    <row r="26" ht="75" customHeight="1">
-      <c r="A26" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-027</t>
-        </is>
-      </c>
-      <c r="B26" s="21" t="inlineStr">
+    <row r="25" ht="75" customHeight="1">
+      <c r="A25" s="26" t="inlineStr">
+        <is>
+          <t>TC-M01-024</t>
+        </is>
+      </c>
+      <c r="B25" s="26" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C26" s="22" t="inlineStr">
+      <c r="C25" s="27" t="inlineStr">
         <is>
           <t>M01-F09</t>
         </is>
       </c>
-      <c r="D26" s="23" t="inlineStr">
+      <c r="D25" s="28" t="inlineStr">
         <is>
           <t>Search &amp; Filter</t>
         </is>
       </c>
-      <c r="E26" s="23" t="inlineStr">
+      <c r="E25" s="28" t="inlineStr">
         <is>
           <t>Search Student by Name Real-time</t>
         </is>
       </c>
-      <c r="F26" s="23" t="inlineStr">
+      <c r="F25" s="28" t="inlineStr">
         <is>
           <t>Verify that searching student list by name filters records dynamically in real-time as the user types.</t>
         </is>
       </c>
-      <c r="G26" s="23" t="inlineStr">
+      <c r="G25" s="28" t="inlineStr">
         <is>
           <t>Staff user is logged in. Student list contains 'Nguyen Van A' and 'Tran Thi B'.</t>
         </is>
       </c>
-      <c r="H26" s="23" t="inlineStr">
+      <c r="H25" s="28" t="inlineStr">
         <is>
           <t>SearchQuery=Nguyen</t>
         </is>
       </c>
-      <c r="I26" s="23" t="inlineStr">
+      <c r="I25" s="28" t="inlineStr">
         <is>
           <t>1. Navigate to student list;
 2. Place cursor in Search box and type 'Nguyen';
 3. Observe student list</t>
         </is>
       </c>
-      <c r="J26" s="23" t="inlineStr">
+      <c r="J25" s="28" t="inlineStr">
         <is>
           <t>The student list filters dynamically while typing. Tran Thi B is hidden, and Nguyen Van A remains visible. No page reload occurs.</t>
         </is>
       </c>
-      <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M26" s="29" t="inlineStr">
+      <c r="K25" s="28" t="inlineStr">
+        <is>
+          <t>The student list filters dynamically while typing. Tran Thi B is hidden, and Nguyen Van A remains visible. No page reload occurs.</t>
+        </is>
+      </c>
+      <c r="L25" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M25" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N26" s="23" t="inlineStr">
+      <c r="N25" s="28" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F09, Scenario: BS-09</t>
         </is>
       </c>
     </row>
-    <row r="27" ht="90" customHeight="1">
-      <c r="A27" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-028</t>
-        </is>
-      </c>
-      <c r="B27" s="26" t="inlineStr">
+    <row r="26" ht="105" customHeight="1">
+      <c r="A26" s="21" t="inlineStr">
+        <is>
+          <t>TC-M01-025</t>
+        </is>
+      </c>
+      <c r="B26" s="21" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C27" s="27" t="inlineStr">
+      <c r="C26" s="22" t="inlineStr">
         <is>
           <t>M01-F09</t>
         </is>
       </c>
-      <c r="D27" s="28" t="inlineStr">
+      <c r="D26" s="23" t="inlineStr">
         <is>
           <t>Search &amp; Filter</t>
         </is>
       </c>
-      <c r="E27" s="28" t="inlineStr">
-        <is>
-          <t>Filter Students by Observation Rating</t>
-        </is>
-      </c>
-      <c r="F27" s="28" t="inlineStr">
-        <is>
-          <t>Verify that staff can filter students by their observation rating.</t>
-        </is>
-      </c>
-      <c r="G27" s="28" t="inlineStr">
-        <is>
-          <t>Staff user is logged in. Students exist with different observation ratings.</t>
-        </is>
-      </c>
-      <c r="H27" s="28" t="inlineStr">
-        <is>
-          <t>RatingFilter=Good</t>
-        </is>
-      </c>
-      <c r="I27" s="28" t="inlineStr">
-        <is>
-          <t>1. Open student list;
-2. Click the Observation Rating filter dropdown;
-3. Choose Good;
-4. Observe the filtered list</t>
-        </is>
-      </c>
-      <c r="J27" s="28" t="inlineStr">
-        <is>
-          <t>The student list is filtered to display only students with a "Good" rating. Other students are hidden.</t>
-        </is>
-      </c>
-      <c r="K27" s="28" t="inlineStr"/>
-      <c r="L27" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M27" s="29" t="inlineStr">
-        <is>
-          <t>Medium</t>
-        </is>
-      </c>
-      <c r="N27" s="28" t="inlineStr">
-        <is>
-          <t>Related Requirement: M01-F09, Scenario: BS-09</t>
-        </is>
-      </c>
-    </row>
-    <row r="28" ht="105" customHeight="1">
-      <c r="A28" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-029</t>
-        </is>
-      </c>
-      <c r="B28" s="21" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="C28" s="22" t="inlineStr">
-        <is>
-          <t>M01-F09</t>
-        </is>
-      </c>
-      <c r="D28" s="23" t="inlineStr">
-        <is>
-          <t>Search &amp; Filter</t>
-        </is>
-      </c>
-      <c r="E28" s="23" t="inlineStr">
+      <c r="E26" s="23" t="inlineStr">
         <is>
           <t>Verify Student List Default Pagination</t>
         </is>
       </c>
-      <c r="F28" s="23" t="inlineStr">
+      <c r="F26" s="23" t="inlineStr">
         <is>
           <t>Verify that the student list displays exactly 10 students per page by default.</t>
         </is>
       </c>
-      <c r="G28" s="23" t="inlineStr">
+      <c r="G26" s="23" t="inlineStr">
         <is>
           <t>Staff user is logged in. There are 12 students in the selected batch.</t>
         </is>
       </c>
-      <c r="H28" s="23" t="inlineStr">
+      <c r="H26" s="23" t="inlineStr">
         <is>
           <t>Batch PNV26A has 12 students.</t>
         </is>
       </c>
-      <c r="I28" s="23" t="inlineStr">
+      <c r="I26" s="23" t="inlineStr">
         <is>
           <t>1. Navigate to the student list of batch PNV26A;
 2. Count the number of students displayed on the first page;
@@ -9310,769 +9262,589 @@
 4. Click Next Page</t>
         </is>
       </c>
-      <c r="J28" s="23" t="inlineStr">
+      <c r="J26" s="23" t="inlineStr">
         <is>
           <t>Page 1 displays exactly 10 students. Pagination controls are visible. Clicking Next Page shows the remaining 2 students on page 2.</t>
         </is>
       </c>
-      <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M28" s="29" t="inlineStr">
+      <c r="K26" s="23" t="inlineStr">
+        <is>
+          <t>Page 1 displays exactly 10 students. Pagination controls are visible. Clicking Next Page shows the remaining 2 students on page 2.</t>
+        </is>
+      </c>
+      <c r="L26" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M26" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N28" s="23" t="inlineStr">
+      <c r="N26" s="23" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F09, Scenario: BS-10</t>
         </is>
       </c>
     </row>
-    <row r="29" ht="75" customHeight="1">
-      <c r="A29" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-030</t>
-        </is>
-      </c>
-      <c r="B29" s="26" t="inlineStr">
+    <row r="27" ht="75" customHeight="1">
+      <c r="A27" s="26" t="inlineStr">
+        <is>
+          <t>TC-M01-026</t>
+        </is>
+      </c>
+      <c r="B27" s="26" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C29" s="27" t="inlineStr">
+      <c r="C27" s="27" t="inlineStr">
         <is>
           <t>M01-F10</t>
         </is>
       </c>
-      <c r="D29" s="28" t="inlineStr">
+      <c r="D27" s="28" t="inlineStr">
         <is>
           <t>Dashboard Overview</t>
         </is>
       </c>
-      <c r="E29" s="28" t="inlineStr">
+      <c r="E27" s="28" t="inlineStr">
         <is>
           <t>Verify Dashboard Displays Correct Initial Stats and Charts</t>
         </is>
       </c>
-      <c r="F29" s="28" t="inlineStr">
+      <c r="F27" s="28" t="inlineStr">
         <is>
           <t>Verify that the dashboard screen accurately loads and displays all student and batch metrics.</t>
         </is>
       </c>
-      <c r="G29" s="28" t="inlineStr">
+      <c r="G27" s="28" t="inlineStr">
         <is>
           <t>Staff user is logged in. System has 2 batches (1 Active, 1 Archived) and 5 students (4 Active, 1 Inactive).</t>
         </is>
       </c>
-      <c r="H29" s="28" t="inlineStr">
+      <c r="H27" s="28" t="inlineStr">
         <is>
           <t>None</t>
         </is>
       </c>
-      <c r="I29" s="28" t="inlineStr">
+      <c r="I27" s="28" t="inlineStr">
         <is>
           <t>1. Navigate to the Dashboard Overview page;
 2. Observe the statistics cards and charts</t>
         </is>
       </c>
-      <c r="J29" s="28" t="inlineStr">
+      <c r="J27" s="28" t="inlineStr">
         <is>
           <t>The dashboard displays: Total Batches = 2, Active Batches = 1, Total Students = 5, Active Students = 4, Inactive Students = 1. Charts (Gender, Ethnicity, Status) load successfully.</t>
         </is>
       </c>
-      <c r="K29" s="28" t="inlineStr"/>
-      <c r="L29" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M29" s="29" t="inlineStr">
+      <c r="K27" s="28" t="inlineStr">
+        <is>
+          <t>The dashboard displays: Total Batches = 2, Active Batches = 1, Total Students = 5, Active Students = 4, Inactive Students = 1. Charts (Gender, Ethnicity, Status) load successfully.</t>
+        </is>
+      </c>
+      <c r="L27" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M27" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N29" s="28" t="inlineStr">
+      <c r="N27" s="28" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F10, Scenario: BS-11</t>
         </is>
       </c>
     </row>
-    <row r="30" ht="90" customHeight="1">
-      <c r="A30" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-031</t>
-        </is>
-      </c>
-      <c r="B30" s="21" t="inlineStr">
+    <row r="28" ht="90" customHeight="1">
+      <c r="A28" s="21" t="inlineStr">
+        <is>
+          <t>TC-M01-027</t>
+        </is>
+      </c>
+      <c r="B28" s="21" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C30" s="22" t="inlineStr">
+      <c r="C28" s="22" t="inlineStr">
         <is>
           <t>M01-F10</t>
         </is>
       </c>
-      <c r="D30" s="23" t="inlineStr">
+      <c r="D28" s="23" t="inlineStr">
         <is>
           <t>Dashboard Overview</t>
         </is>
       </c>
-      <c r="E30" s="23" t="inlineStr">
+      <c r="E28" s="23" t="inlineStr">
         <is>
           <t>Verify Dashboard Stats Auto-refresh after Data Changes</t>
         </is>
       </c>
-      <c r="F30" s="23" t="inlineStr">
+      <c r="F28" s="23" t="inlineStr">
         <is>
           <t>Verify that dashboard statistics and charts refresh automatically when data changes.</t>
         </is>
       </c>
-      <c r="G30" s="23" t="inlineStr">
+      <c r="G28" s="23" t="inlineStr">
         <is>
           <t>Staff user is logged in. Dashboard shows Active Students = 4.</t>
         </is>
       </c>
-      <c r="H30" s="23" t="inlineStr">
+      <c r="H28" s="23" t="inlineStr">
         <is>
           <t>StudentCode=ST001; NewStatus=Inactive</t>
         </is>
       </c>
-      <c r="I30" s="23" t="inlineStr">
+      <c r="I28" s="23" t="inlineStr">
         <is>
           <t>1. Navigate to student list and edit ST001 to change status from Active to Inactive;
 2. Click Save;
 3. Immediately return to the Dashboard</t>
         </is>
       </c>
-      <c r="J30" s="23" t="inlineStr">
+      <c r="J28" s="23" t="inlineStr">
         <is>
           <t>The dashboard values update without manual page reload: Active Students displays 3, Inactive Students displays 2, and charts adjust accordingly.</t>
         </is>
       </c>
-      <c r="K30" s="23" t="inlineStr"/>
-      <c r="L30" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M30" s="29" t="inlineStr">
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>The dashboard values update without manual page reload: Active Students displays 3, Inactive Students displays 2, and charts adjust accordingly.</t>
+        </is>
+      </c>
+      <c r="L28" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M28" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N30" s="23" t="inlineStr">
+      <c r="N28" s="23" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F10, Scenario: BS-11</t>
         </is>
       </c>
     </row>
-    <row r="31" ht="60" customHeight="1">
-      <c r="A31" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-032</t>
-        </is>
-      </c>
-      <c r="B31" s="26" t="inlineStr">
+    <row r="29" ht="60" customHeight="1">
+      <c r="A29" s="26" t="inlineStr">
+        <is>
+          <t>TC-M01-028</t>
+        </is>
+      </c>
+      <c r="B29" s="26" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C31" s="27" t="inlineStr">
+      <c r="C29" s="27" t="inlineStr">
         <is>
           <t>M01-SEC</t>
         </is>
       </c>
-      <c r="D31" s="28" t="inlineStr">
+      <c r="D29" s="28" t="inlineStr">
         <is>
           <t>Access Control &amp; Security</t>
         </is>
       </c>
-      <c r="E31" s="28" t="inlineStr">
+      <c r="E29" s="28" t="inlineStr">
         <is>
           <t>Staff User Access to Student Management</t>
         </is>
       </c>
-      <c r="F31" s="28" t="inlineStr">
+      <c r="F29" s="28" t="inlineStr">
         <is>
           <t>Verify that staff users with a valid @passerellesnumeriques.org email domain are granted access to Batch &amp; Student Management.</t>
         </is>
       </c>
-      <c r="G31" s="28" t="inlineStr">
+      <c r="G29" s="28" t="inlineStr">
         <is>
           <t>User is authenticated with email staff@passerellesnumeriques.org.</t>
         </is>
       </c>
-      <c r="H31" s="28" t="inlineStr">
+      <c r="H29" s="28" t="inlineStr">
         <is>
           <t>Email=staff@passerellesnumeriques.org</t>
         </is>
       </c>
-      <c r="I31" s="28" t="inlineStr">
+      <c r="I29" s="28" t="inlineStr">
         <is>
           <t>1. Enter the application URL;
 2. Sign in via Google OAuth with account staff@passerellesnumeriques.org</t>
         </is>
       </c>
-      <c r="J31" s="28" t="inlineStr">
+      <c r="J29" s="28" t="inlineStr">
         <is>
           <t>The user is redirected to the Staff Portal. Full management options (Create Batch, Add Student, Edit, CSV Import) are visible and accessible.</t>
         </is>
       </c>
-      <c r="K31" s="28" t="inlineStr"/>
-      <c r="L31" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M31" s="25" t="inlineStr">
+      <c r="K29" s="28" t="inlineStr">
+        <is>
+          <t>The user is redirected to the Staff Portal. Full management options (Create Batch, Add Student, Edit, CSV Import) are visible and accessible.</t>
+        </is>
+      </c>
+      <c r="L29" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M29" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N31" s="28" t="inlineStr">
+      <c r="N29" s="28" t="inlineStr">
         <is>
           <t>Related Requirement: General Business Rules, Scenario: BS-12</t>
         </is>
       </c>
     </row>
-    <row r="32" ht="60" customHeight="1">
-      <c r="A32" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-033</t>
-        </is>
-      </c>
-      <c r="B32" s="21" t="inlineStr">
+    <row r="30" ht="60" customHeight="1">
+      <c r="A30" s="21" t="inlineStr">
+        <is>
+          <t>TC-M01-029</t>
+        </is>
+      </c>
+      <c r="B30" s="21" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C32" s="22" t="inlineStr">
+      <c r="C30" s="22" t="inlineStr">
         <is>
           <t>M01-SEC</t>
         </is>
       </c>
-      <c r="D32" s="23" t="inlineStr">
+      <c r="D30" s="23" t="inlineStr">
         <is>
           <t>Access Control &amp; Security</t>
         </is>
       </c>
-      <c r="E32" s="23" t="inlineStr">
+      <c r="E30" s="23" t="inlineStr">
         <is>
           <t>Student User Access to Student Management Denied</t>
         </is>
       </c>
-      <c r="F32" s="23" t="inlineStr">
+      <c r="F30" s="23" t="inlineStr">
         <is>
           <t>Verify that students with a @student.passerellesnumeriques.org email are denied management access.</t>
         </is>
       </c>
-      <c r="G32" s="23" t="inlineStr">
+      <c r="G30" s="23" t="inlineStr">
         <is>
           <t>User is authenticated with email student01@student.passerellesnumeriques.org.</t>
         </is>
       </c>
-      <c r="H32" s="23" t="inlineStr">
+      <c r="H30" s="23" t="inlineStr">
         <is>
           <t>Email=student01@student.passerellesnumeriques.org</t>
         </is>
       </c>
-      <c r="I32" s="23" t="inlineStr">
+      <c r="I30" s="23" t="inlineStr">
         <is>
           <t>1. Enter the application URL;
 2. Sign in via Google OAuth with account student01@student.passerellesnumeriques.org</t>
         </is>
       </c>
-      <c r="J32" s="23" t="inlineStr">
+      <c r="J30" s="23" t="inlineStr">
         <is>
           <t>The user is redirected to the Student Portal. Management buttons and options are hidden. Direct URL routing to staff pages displays "Access Denied".</t>
         </is>
       </c>
-      <c r="K32" s="23" t="inlineStr"/>
-      <c r="L32" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M32" s="25" t="inlineStr">
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>The user is redirected to the Student Portal. Management buttons and options are hidden. Direct URL routing to staff pages displays "Access Denied".</t>
+        </is>
+      </c>
+      <c r="L30" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M30" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N32" s="23" t="inlineStr">
+      <c r="N30" s="23" t="inlineStr">
         <is>
           <t>Related Requirement: General Business Rules, Scenario: BS-12</t>
         </is>
       </c>
     </row>
-    <row r="33" ht="90" customHeight="1">
-      <c r="A33" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-018</t>
-        </is>
-      </c>
-      <c r="B33" s="26" t="inlineStr">
+    <row r="31" ht="90" customHeight="1">
+      <c r="A31" s="26" t="inlineStr">
+        <is>
+          <t>TC-M01-030</t>
+        </is>
+      </c>
+      <c r="B31" s="26" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C33" s="27" t="inlineStr">
-        <is>
-          <t>M01-F05</t>
-        </is>
-      </c>
-      <c r="D33" s="28" t="inlineStr">
-        <is>
-          <t>Bulk Student Import</t>
-        </is>
-      </c>
-      <c r="E33" s="28" t="inlineStr">
-        <is>
-          <t>CSV Student Import Upsert</t>
-        </is>
-      </c>
-      <c r="F33" s="28" t="inlineStr">
-        <is>
-          <t>Verify that bulk student import via CSV updates existing profiles and creates new profiles (Upsert behavior).</t>
-        </is>
-      </c>
-      <c r="G33" s="28" t="inlineStr">
-        <is>
-          <t>Staff user is logged in. Student ST001 already exists; batch PNV26A exists.</t>
-        </is>
-      </c>
-      <c r="H33" s="28" t="inlineStr">
-        <is>
-          <t>CSV row: ST001,Nguyen Van A Updated,2006-05-15,Male,nguyenvana.new@student.passerellesnumeriques.org,AssociatedBatch=PNV26A and ST003,Le Van C,2006-08-20,Male,levanc.st26@student.passerellesnumeriques.org,AssociatedBatch=PNV26A</t>
-        </is>
-      </c>
-      <c r="I33" s="28" t="inlineStr">
-        <is>
-          <t>1. Go to CSV Import page;
-2. Upload CSV containing update row for ST001 and new row for ST003;
-3. Click Import</t>
-        </is>
-      </c>
-      <c r="J33" s="28" t="inlineStr">
-        <is>
-          <t>Import completes successfully. Message displays "Import successful. 1 student updated, 1 student created.". ST001 displays new name and ST003 appears in list.</t>
-        </is>
-      </c>
-      <c r="K33" s="28" t="inlineStr"/>
-      <c r="L33" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M33" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="N33" s="28" t="inlineStr">
-        <is>
-          <t>Related Requirement: M01-F05, Scenario: BS-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="34" ht="60" customHeight="1">
-      <c r="A34" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-019</t>
-        </is>
-      </c>
-      <c r="B34" s="21" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="C34" s="22" t="inlineStr">
-        <is>
-          <t>M01-F05</t>
-        </is>
-      </c>
-      <c r="D34" s="23" t="inlineStr">
-        <is>
-          <t>Bulk Student Import</t>
-        </is>
-      </c>
-      <c r="E34" s="23" t="inlineStr">
-        <is>
-          <t>CSV Student Import Rejects Duplicate Student Codes</t>
-        </is>
-      </c>
-      <c r="F34" s="23" t="inlineStr">
-        <is>
-          <t>Verify that student bulk import via CSV rejects imports with duplicate student codes within the file.</t>
-        </is>
-      </c>
-      <c r="G34" s="23" t="inlineStr">
-        <is>
-          <t>Staff user is logged in.</t>
-        </is>
-      </c>
-      <c r="H34" s="23" t="inlineStr">
-        <is>
-          <t>CSV containing two rows with student code ST004</t>
-        </is>
-      </c>
-      <c r="I34" s="23" t="inlineStr">
-        <is>
-          <t>1. Go to CSV Import page;
-2. Upload CSV with duplicate ST004;
-3. Click Import</t>
-        </is>
-      </c>
-      <c r="J34" s="23" t="inlineStr">
-        <is>
-          <t>The system rejects the entire CSV file. Error message appears: "Duplicate student code: ST004.". No records are imported.</t>
-        </is>
-      </c>
-      <c r="K34" s="23" t="inlineStr"/>
-      <c r="L34" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M34" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="N34" s="23" t="inlineStr">
-        <is>
-          <t>Related Requirement: M01-F05, Scenario: BS-05</t>
-        </is>
-      </c>
-    </row>
-    <row r="35" ht="90" customHeight="1">
-      <c r="A35" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-034</t>
-        </is>
-      </c>
-      <c r="B35" s="26" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="C35" s="27" t="inlineStr">
+      <c r="C31" s="27" t="inlineStr">
         <is>
           <t>M01-SEC</t>
         </is>
       </c>
-      <c r="D35" s="28" t="inlineStr">
+      <c r="D31" s="28" t="inlineStr">
         <is>
           <t>Access Control &amp; Security</t>
         </is>
       </c>
-      <c r="E35" s="28" t="inlineStr">
+      <c r="E31" s="28" t="inlineStr">
         <is>
           <t>Unknown Email Domain Access Denied</t>
         </is>
       </c>
-      <c r="F35" s="28" t="inlineStr">
+      <c r="F31" s="28" t="inlineStr">
         <is>
           <t>Verify that users with non-permitted email domains are completely blocked from accessing the system.</t>
         </is>
       </c>
-      <c r="G35" s="28" t="inlineStr">
+      <c r="G31" s="28" t="inlineStr">
         <is>
           <t>User is authenticated with email testuser@gmail.com.</t>
         </is>
       </c>
-      <c r="H35" s="28" t="inlineStr">
+      <c r="H31" s="28" t="inlineStr">
         <is>
           <t>Email=testuser@gmail.com</t>
         </is>
       </c>
-      <c r="I35" s="28" t="inlineStr">
+      <c r="I31" s="28" t="inlineStr">
         <is>
           <t>1. Enter the application URL;
 2. Sign in via Google OAuth with account testuser@gmail.com;
 3. Observe the system response</t>
         </is>
       </c>
-      <c r="J35" s="28" t="inlineStr">
-        <is>
-          <t>Login fails or the screen displays an "Access Denied" message. The user is not redirected to either the Staff or Student Portal.</t>
-        </is>
-      </c>
-      <c r="K35" s="28" t="inlineStr"/>
-      <c r="L35" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M35" s="25" t="inlineStr">
+      <c r="J31" s="28" t="inlineStr">
+        <is>
+          <t>Login failed, or the screen displays a notification stating that this page cannot be accessed.</t>
+        </is>
+      </c>
+      <c r="K31" s="28" t="inlineStr">
+        <is>
+          <t>Login failed, or the screen displays a notification stating that this page cannot be accessed.</t>
+        </is>
+      </c>
+      <c r="L31" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M31" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N35" s="28" t="inlineStr">
+      <c r="N31" s="28" t="inlineStr">
         <is>
           <t>Related Requirement: General Business Rules, Authorization</t>
         </is>
       </c>
     </row>
-    <row r="36" ht="135" customHeight="1">
-      <c r="A36" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-035</t>
-        </is>
-      </c>
-      <c r="B36" s="21" t="inlineStr">
+    <row r="32" ht="75" customHeight="1">
+      <c r="A32" s="21" t="inlineStr">
+        <is>
+          <t>TC-M01-031</t>
+        </is>
+      </c>
+      <c r="B32" s="21" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C36" s="22" t="inlineStr">
-        <is>
-          <t>M01-F04</t>
-        </is>
-      </c>
-      <c r="D36" s="23" t="inlineStr">
-        <is>
-          <t>Single Student Creation</t>
-        </is>
-      </c>
-      <c r="E36" s="23" t="inlineStr">
-        <is>
-          <t>Create Student Fails due to Missing Associated Batch</t>
-        </is>
-      </c>
-      <c r="F36" s="23" t="inlineStr">
-        <is>
-          <t>Verify that manually creating a student requires selecting an Associated Batch.</t>
-        </is>
-      </c>
-      <c r="G36" s="23" t="inlineStr">
+      <c r="C32" s="22" t="inlineStr">
+        <is>
+          <t>M01-F05</t>
+        </is>
+      </c>
+      <c r="D32" s="23" t="inlineStr">
+        <is>
+          <t>Bulk Student Import</t>
+        </is>
+      </c>
+      <c r="E32" s="23" t="inlineStr">
+        <is>
+          <t>CSV Student Import Fails due to Blank Name</t>
+        </is>
+      </c>
+      <c r="F32" s="23" t="inlineStr">
+        <is>
+          <t>Verify that bulk import via CSV blocks saving if student name is empty.</t>
+        </is>
+      </c>
+      <c r="G32" s="23" t="inlineStr">
         <is>
           <t>Staff user is logged in.</t>
         </is>
       </c>
-      <c r="H36" s="23" t="inlineStr">
-        <is>
-          <t>StudentCode=ST099; StudentName=Nguyen Van Test; AssociatedBatch=Empty</t>
-        </is>
-      </c>
-      <c r="I36" s="23" t="inlineStr">
-        <is>
-          <t>1. Open Batch Management;
-2. Click Add Student;
-3. Enter Student Code 'ST099' and Name 'Nguyen Van Test';
-4. Leave Associated Batch selection empty;
-5. Click Save</t>
-        </is>
-      </c>
-      <c r="J36" s="23" t="inlineStr">
-        <is>
-          <t>The system blocks saving and displays a validation error "Associated Batch is required". The batch dropdown is highlighted in red.</t>
-        </is>
-      </c>
-      <c r="K36" s="23" t="inlineStr"/>
-      <c r="L36" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M36" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="N36" s="23" t="inlineStr">
-        <is>
-          <t>Related Requirement: M01-F04, Validation Rules</t>
-        </is>
-      </c>
-    </row>
-    <row r="37" ht="75" customHeight="1">
-      <c r="A37" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-036</t>
-        </is>
-      </c>
-      <c r="B37" s="26" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="C37" s="27" t="inlineStr">
-        <is>
-          <t>M01-F05</t>
-        </is>
-      </c>
-      <c r="D37" s="28" t="inlineStr">
-        <is>
-          <t>Bulk Student Import</t>
-        </is>
-      </c>
-      <c r="E37" s="28" t="inlineStr">
-        <is>
-          <t>CSV Student Import Fails due to Blank Name</t>
-        </is>
-      </c>
-      <c r="F37" s="28" t="inlineStr">
-        <is>
-          <t>Verify that bulk import via CSV blocks saving if student name is empty.</t>
-        </is>
-      </c>
-      <c r="G37" s="28" t="inlineStr">
-        <is>
-          <t>Staff user is logged in.</t>
-        </is>
-      </c>
-      <c r="H37" s="28" t="inlineStr">
+      <c r="H32" s="23" t="inlineStr">
         <is>
           <t>CSV contains row: ST006,,2006-08-20,Male,student06@student.passerellesnumeriques.org (blank name)</t>
         </is>
       </c>
-      <c r="I37" s="28" t="inlineStr">
+      <c r="I32" s="23" t="inlineStr">
         <is>
           <t>1. Go to CSV Import page;
 2. Upload the CSV file with blank name;
 3. Click Import</t>
         </is>
       </c>
-      <c r="J37" s="28" t="inlineStr">
+      <c r="J32" s="23" t="inlineStr">
         <is>
           <t>The system rejects the entire CSV file with error message "Student Name is required". No records are updated in database.</t>
         </is>
       </c>
-      <c r="K37" s="28" t="inlineStr"/>
-      <c r="L37" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M37" s="25" t="inlineStr">
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>The system rejects the entire CSV file with error message "Student Name is required". No records are updated in database.</t>
+        </is>
+      </c>
+      <c r="L32" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M32" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N37" s="28" t="inlineStr">
+      <c r="N32" s="23" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F05, Validation Rules</t>
         </is>
       </c>
     </row>
-    <row r="38" ht="75" customHeight="1">
-      <c r="A38" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-037</t>
-        </is>
-      </c>
-      <c r="B38" s="21" t="inlineStr">
+    <row r="33" ht="75" customHeight="1">
+      <c r="A33" s="26" t="inlineStr">
+        <is>
+          <t>TC-M01-032</t>
+        </is>
+      </c>
+      <c r="B33" s="26" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C38" s="22" t="inlineStr">
+      <c r="C33" s="27" t="inlineStr">
         <is>
           <t>M01-F09</t>
         </is>
       </c>
-      <c r="D38" s="23" t="inlineStr">
+      <c r="D33" s="28" t="inlineStr">
         <is>
           <t>Search &amp; Filter</t>
         </is>
       </c>
-      <c r="E38" s="23" t="inlineStr">
+      <c r="E33" s="28" t="inlineStr">
         <is>
           <t>Search Student Case Insensitivity</t>
         </is>
       </c>
-      <c r="F38" s="23" t="inlineStr">
+      <c r="F33" s="28" t="inlineStr">
         <is>
           <t>Verify that student search filters correctly regardless of character casing.</t>
         </is>
       </c>
-      <c r="G38" s="23" t="inlineStr">
+      <c r="G33" s="28" t="inlineStr">
         <is>
           <t>Staff user is logged in. Batch PNV26A contains student 'Nguyen Van A'.</t>
         </is>
       </c>
-      <c r="H38" s="23" t="inlineStr">
+      <c r="H33" s="28" t="inlineStr">
         <is>
           <t>SearchQuery=nguyen van a</t>
         </is>
       </c>
-      <c r="I38" s="23" t="inlineStr">
+      <c r="I33" s="28" t="inlineStr">
         <is>
           <t>1. Open student list;
 2. Enter 'nguyen van a' (all lowercase) in the search box;
 3. Verify matching result</t>
         </is>
       </c>
-      <c r="J38" s="23" t="inlineStr">
+      <c r="J33" s="28" t="inlineStr">
         <is>
           <t>The student list filters and displays 'Nguyen Van A', proving search is case-insensitive.</t>
         </is>
       </c>
-      <c r="K38" s="23" t="inlineStr"/>
-      <c r="L38" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M38" s="29" t="inlineStr">
+      <c r="K33" s="28" t="inlineStr">
+        <is>
+          <t>The student list filters and displays 'Nguyen Van A', proving search is case-insensitive.</t>
+        </is>
+      </c>
+      <c r="L33" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
+        </is>
+      </c>
+      <c r="M33" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
         </is>
       </c>
-      <c r="N38" s="23" t="inlineStr">
+      <c r="N33" s="28" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F09, Search &amp; Filter</t>
         </is>
       </c>
     </row>
-    <row r="39" ht="90" customHeight="1">
-      <c r="A39" s="26" t="inlineStr">
-        <is>
-          <t>TC-M01-038</t>
-        </is>
-      </c>
-      <c r="B39" s="26" t="inlineStr">
+    <row r="34" ht="90" customHeight="1">
+      <c r="A34" s="21" t="inlineStr">
+        <is>
+          <t>TC-M01-033</t>
+        </is>
+      </c>
+      <c r="B34" s="21" t="inlineStr">
         <is>
           <t>Module 01</t>
         </is>
       </c>
-      <c r="C39" s="27" t="inlineStr">
+      <c r="C34" s="22" t="inlineStr">
         <is>
           <t>M01-F06</t>
         </is>
       </c>
-      <c r="D39" s="28" t="inlineStr">
+      <c r="D34" s="23" t="inlineStr">
         <is>
           <t>Student Editing</t>
         </is>
       </c>
-      <c r="E39" s="28" t="inlineStr">
+      <c r="E34" s="23" t="inlineStr">
         <is>
           <t>Edit Student Email to Invalid Format Blocked</t>
         </is>
       </c>
-      <c r="F39" s="28" t="inlineStr">
+      <c r="F34" s="23" t="inlineStr">
         <is>
           <t>Verify that editing a student's email to an invalid format is blocked.</t>
         </is>
       </c>
-      <c r="G39" s="28" t="inlineStr">
+      <c r="G34" s="23" t="inlineStr">
         <is>
           <t>Staff user is logged in. Student ST001 exists.</t>
         </is>
       </c>
-      <c r="H39" s="28" t="inlineStr">
+      <c r="H34" s="23" t="inlineStr">
         <is>
           <t>StudentCode=ST001; NewEmail=nguyenvana_invalid_email</t>
         </is>
       </c>
-      <c r="I39" s="28" t="inlineStr">
+      <c r="I34" s="23" t="inlineStr">
         <is>
           <t>1. Open student list;
 2. Select ST001 and click Edit;
@@ -10080,105 +9852,39 @@
 4. Click Save</t>
         </is>
       </c>
-      <c r="J39" s="28" t="inlineStr">
+      <c r="J34" s="23" t="inlineStr">
         <is>
           <t>The system blocks saving and displays a validation error message requiring a valid email format. The email field is highlighted in red.</t>
         </is>
       </c>
-      <c r="K39" s="28" t="inlineStr"/>
-      <c r="L39" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M39" s="25" t="inlineStr">
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>The system successfully updated the email address, even though the format was incorrect.</t>
+        </is>
+      </c>
+      <c r="L34" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="M34" s="25" t="inlineStr">
         <is>
           <t>High</t>
         </is>
       </c>
-      <c r="N39" s="28" t="inlineStr">
+      <c r="N34" s="23" t="inlineStr">
         <is>
           <t>Related Requirement: M01-F06, Validation Rules</t>
         </is>
       </c>
     </row>
-    <row r="40" ht="75" customHeight="1">
-      <c r="A40" s="21" t="inlineStr">
-        <is>
-          <t>TC-M01-039</t>
-        </is>
-      </c>
-      <c r="B40" s="21" t="inlineStr">
-        <is>
-          <t>Module 01</t>
-        </is>
-      </c>
-      <c r="C40" s="22" t="inlineStr">
-        <is>
-          <t>M01-F05</t>
-        </is>
-      </c>
-      <c r="D40" s="23" t="inlineStr">
-        <is>
-          <t>Bulk Student Import</t>
-        </is>
-      </c>
-      <c r="E40" s="23" t="inlineStr">
-        <is>
-          <t>CSV Student Import Blocked due to Duplicate Student Code in Another Batch</t>
-        </is>
-      </c>
-      <c r="F40" s="23" t="inlineStr">
-        <is>
-          <t>Verify that CSV student import rejects student codes that are already in use in other batches.</t>
-        </is>
-      </c>
-      <c r="G40" s="23" t="inlineStr">
-        <is>
-          <t>Student ST001 exists in batch PNV26A. Batch PNV26B has no students.</t>
-        </is>
-      </c>
-      <c r="H40" s="23" t="inlineStr">
-        <is>
-          <t>CSV file for batch PNV26B containing row: ST001,Le Van C,2006-08-20,Male,levanc.st26@student.passerellesnumeriques.org</t>
-        </is>
-      </c>
-      <c r="I40" s="23" t="inlineStr">
-        <is>
-          <t>1. Go to CSV Import page for batch PNV26B;
-2. Upload CSV containing student ST001;
-3. Click Import</t>
-        </is>
-      </c>
-      <c r="J40" s="23" t="inlineStr">
-        <is>
-          <t>The system rejects the import and displays error message "Duplicate student code: ST001.". No students are added.</t>
-        </is>
-      </c>
-      <c r="K40" s="23" t="inlineStr"/>
-      <c r="L40" s="24" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M40" s="25" t="inlineStr">
-        <is>
-          <t>High</t>
-        </is>
-      </c>
-      <c r="N40" s="23" t="inlineStr">
-        <is>
-          <t>Related Requirement: M01-F05, Student Code Uniqueness</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:N40"/>
+  <autoFilter ref="A1:N34"/>
   <dataValidations count="2">
-    <dataValidation sqref="L2:L140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Status" error="Please select a valid state: Passed, Failed, or Not Run" type="list">
+    <dataValidation sqref="L2:L134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Status" error="Please select a valid state: Passed, Failed, or Not Run" type="list">
       <formula1>"Passed,Failed,Not Run"</formula1>
     </dataValidation>
-    <dataValidation sqref="M2:M140" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Priority" error="Please select a valid priority: High, Medium, or Low" type="list">
+    <dataValidation sqref="M2:M134" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" errorTitle="Invalid Priority" error="Please select a valid priority: High, Medium, or Low" type="list">
       <formula1>"High,Medium,Low"</formula1>
     </dataValidation>
   </dataValidations>
@@ -10342,7 +10048,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
+      <c r="L2" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10414,7 +10120,7 @@
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10486,7 +10192,7 @@
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10557,7 +10263,7 @@
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10628,7 +10334,7 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10699,7 +10405,7 @@
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10770,7 +10476,7 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10841,7 +10547,7 @@
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10912,7 +10618,7 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -10981,7 +10687,7 @@
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11050,7 +10756,7 @@
         </is>
       </c>
       <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11120,7 +10826,7 @@
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11190,7 +10896,7 @@
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11260,7 +10966,7 @@
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11331,7 +11037,7 @@
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11402,7 +11108,7 @@
         </is>
       </c>
       <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
+      <c r="L17" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11472,7 +11178,7 @@
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
+      <c r="L18" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11543,7 +11249,7 @@
         </is>
       </c>
       <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="L19" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11615,7 +11321,7 @@
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11684,7 +11390,7 @@
         </is>
       </c>
       <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
+      <c r="L21" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11754,7 +11460,7 @@
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
+      <c r="L22" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11826,7 +11532,7 @@
         </is>
       </c>
       <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
+      <c r="L23" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11898,7 +11604,7 @@
         </is>
       </c>
       <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
+      <c r="L24" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -11970,7 +11676,7 @@
         </is>
       </c>
       <c r="K25" s="28" t="inlineStr"/>
-      <c r="L25" s="24" t="inlineStr">
+      <c r="L25" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12042,7 +11748,7 @@
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="24" t="inlineStr">
+      <c r="L26" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12113,7 +11819,7 @@
         </is>
       </c>
       <c r="K27" s="28" t="inlineStr"/>
-      <c r="L27" s="24" t="inlineStr">
+      <c r="L27" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12184,7 +11890,7 @@
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr">
+      <c r="L28" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12254,7 +11960,7 @@
         </is>
       </c>
       <c r="K29" s="28" t="inlineStr"/>
-      <c r="L29" s="24" t="inlineStr">
+      <c r="L29" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12324,7 +12030,7 @@
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr"/>
-      <c r="L30" s="24" t="inlineStr">
+      <c r="L30" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12395,7 +12101,7 @@
         </is>
       </c>
       <c r="K31" s="28" t="inlineStr"/>
-      <c r="L31" s="24" t="inlineStr">
+      <c r="L31" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12466,7 +12172,7 @@
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr"/>
-      <c r="L32" s="24" t="inlineStr">
+      <c r="L32" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12649,7 +12355,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
+      <c r="L2" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12720,7 +12426,7 @@
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12792,7 +12498,7 @@
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12864,7 +12570,7 @@
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -12935,7 +12641,7 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13006,7 +12712,7 @@
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13077,7 +12783,7 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13148,7 +12854,7 @@
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13218,7 +12924,7 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13289,7 +12995,7 @@
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13359,7 +13065,7 @@
         </is>
       </c>
       <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13429,7 +13135,7 @@
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13497,7 +13203,7 @@
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13569,7 +13275,7 @@
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13639,7 +13345,7 @@
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13710,7 +13416,7 @@
         </is>
       </c>
       <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
+      <c r="L17" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13781,7 +13487,7 @@
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
+      <c r="L18" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13852,7 +13558,7 @@
         </is>
       </c>
       <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="L19" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13922,7 +13628,7 @@
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -13992,7 +13698,7 @@
         </is>
       </c>
       <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
+      <c r="L21" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14062,7 +13768,7 @@
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
+      <c r="L22" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14132,7 +13838,7 @@
         </is>
       </c>
       <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
+      <c r="L23" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14319,7 +14025,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
+      <c r="L2" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14392,7 +14098,7 @@
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14463,7 +14169,7 @@
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14534,7 +14240,7 @@
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14604,7 +14310,7 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14675,7 +14381,7 @@
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14746,7 +14452,7 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14816,7 +14522,7 @@
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14887,7 +14593,7 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -14958,7 +14664,7 @@
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15029,7 +14735,7 @@
         </is>
       </c>
       <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15100,7 +14806,7 @@
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15170,7 +14876,7 @@
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15239,7 +14945,7 @@
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15308,7 +15014,7 @@
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15379,7 +15085,7 @@
         </is>
       </c>
       <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
+      <c r="L17" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15450,7 +15156,7 @@
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
+      <c r="L18" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15521,7 +15227,7 @@
         </is>
       </c>
       <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="L19" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15592,7 +15298,7 @@
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15662,7 +15368,7 @@
         </is>
       </c>
       <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
+      <c r="L21" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15731,7 +15437,7 @@
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
+      <c r="L22" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15801,7 +15507,7 @@
         </is>
       </c>
       <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
+      <c r="L23" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -15872,7 +15578,7 @@
         </is>
       </c>
       <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
+      <c r="L24" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16059,7 +15765,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
+      <c r="L2" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16135,7 +15841,7 @@
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16210,7 +15916,7 @@
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16285,7 +15991,7 @@
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16360,7 +16066,7 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16434,7 +16140,7 @@
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16505,7 +16211,7 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16578,7 +16284,7 @@
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16651,7 +16357,7 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16724,7 +16430,7 @@
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16796,7 +16502,7 @@
         </is>
       </c>
       <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16869,7 +16575,7 @@
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -16941,7 +16647,7 @@
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17016,7 +16722,7 @@
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17090,7 +16796,7 @@
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17162,7 +16868,7 @@
         </is>
       </c>
       <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
+      <c r="L17" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17234,7 +16940,7 @@
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
+      <c r="L18" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17305,7 +17011,7 @@
         </is>
       </c>
       <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="L19" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17376,7 +17082,7 @@
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17452,7 +17158,7 @@
         </is>
       </c>
       <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
+      <c r="L21" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17528,7 +17234,7 @@
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
+      <c r="L22" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17604,7 +17310,7 @@
         </is>
       </c>
       <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
+      <c r="L23" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17677,7 +17383,7 @@
         </is>
       </c>
       <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
+      <c r="L24" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17751,7 +17457,7 @@
         </is>
       </c>
       <c r="K25" s="28" t="inlineStr"/>
-      <c r="L25" s="24" t="inlineStr">
+      <c r="L25" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17824,7 +17530,7 @@
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="24" t="inlineStr">
+      <c r="L26" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17898,7 +17604,7 @@
         </is>
       </c>
       <c r="K27" s="28" t="inlineStr"/>
-      <c r="L27" s="24" t="inlineStr">
+      <c r="L27" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -17973,7 +17679,7 @@
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr">
+      <c r="L28" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18157,7 +17863,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
+      <c r="L2" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18229,7 +17935,7 @@
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18301,7 +18007,7 @@
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18371,7 +18077,7 @@
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18444,7 +18150,7 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18517,7 +18223,7 @@
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18589,7 +18295,7 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18660,7 +18366,7 @@
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18731,7 +18437,7 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18802,7 +18508,7 @@
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18874,7 +18580,7 @@
         </is>
       </c>
       <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -18945,7 +18651,7 @@
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19017,7 +18723,7 @@
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19088,7 +18794,7 @@
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19158,7 +18864,7 @@
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19228,7 +18934,7 @@
         </is>
       </c>
       <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
+      <c r="L17" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19296,7 +19002,7 @@
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
+      <c r="L18" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19373,7 +19079,7 @@
         </is>
       </c>
       <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="L19" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19443,7 +19149,7 @@
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19513,7 +19219,7 @@
         </is>
       </c>
       <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
+      <c r="L21" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19583,7 +19289,7 @@
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
+      <c r="L22" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19653,7 +19359,7 @@
         </is>
       </c>
       <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
+      <c r="L23" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19723,7 +19429,7 @@
         </is>
       </c>
       <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
+      <c r="L24" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19793,7 +19499,7 @@
         </is>
       </c>
       <c r="K25" s="28" t="inlineStr"/>
-      <c r="L25" s="24" t="inlineStr">
+      <c r="L25" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19863,7 +19569,7 @@
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="24" t="inlineStr">
+      <c r="L26" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -19934,7 +19640,7 @@
         </is>
       </c>
       <c r="K27" s="28" t="inlineStr"/>
-      <c r="L27" s="24" t="inlineStr">
+      <c r="L27" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20006,7 +19712,7 @@
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr">
+      <c r="L28" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20076,7 +19782,7 @@
         </is>
       </c>
       <c r="K29" s="28" t="inlineStr"/>
-      <c r="L29" s="24" t="inlineStr">
+      <c r="L29" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20147,7 +19853,7 @@
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr"/>
-      <c r="L30" s="24" t="inlineStr">
+      <c r="L30" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20218,7 +19924,7 @@
         </is>
       </c>
       <c r="K31" s="28" t="inlineStr"/>
-      <c r="L31" s="24" t="inlineStr">
+      <c r="L31" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20289,7 +19995,7 @@
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr"/>
-      <c r="L32" s="24" t="inlineStr">
+      <c r="L32" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20473,7 +20179,7 @@
         </is>
       </c>
       <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="24" t="inlineStr">
+      <c r="L2" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20544,7 +20250,7 @@
         </is>
       </c>
       <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="24" t="inlineStr">
+      <c r="L3" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20614,7 +20320,7 @@
         </is>
       </c>
       <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="24" t="inlineStr">
+      <c r="L4" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20683,7 +20389,7 @@
         </is>
       </c>
       <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="24" t="inlineStr">
+      <c r="L5" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20756,7 +20462,7 @@
         </is>
       </c>
       <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="24" t="inlineStr">
+      <c r="L6" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20826,7 +20532,7 @@
         </is>
       </c>
       <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="24" t="inlineStr">
+      <c r="L7" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20898,7 +20604,7 @@
         </is>
       </c>
       <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="24" t="inlineStr">
+      <c r="L8" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -20969,7 +20675,7 @@
         </is>
       </c>
       <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="24" t="inlineStr">
+      <c r="L9" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21041,7 +20747,7 @@
         </is>
       </c>
       <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="24" t="inlineStr">
+      <c r="L10" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21111,7 +20817,7 @@
         </is>
       </c>
       <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="24" t="inlineStr">
+      <c r="L11" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21184,7 +20890,7 @@
         </is>
       </c>
       <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="24" t="inlineStr">
+      <c r="L12" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21254,7 +20960,7 @@
         </is>
       </c>
       <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="24" t="inlineStr">
+      <c r="L13" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21325,7 +21031,7 @@
         </is>
       </c>
       <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="24" t="inlineStr">
+      <c r="L14" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21395,7 +21101,7 @@
         </is>
       </c>
       <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="24" t="inlineStr">
+      <c r="L15" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21466,7 +21172,7 @@
         </is>
       </c>
       <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="24" t="inlineStr">
+      <c r="L16" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21534,7 +21240,7 @@
         </is>
       </c>
       <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="24" t="inlineStr">
+      <c r="L17" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21607,7 +21313,7 @@
         </is>
       </c>
       <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="24" t="inlineStr">
+      <c r="L18" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21677,7 +21383,7 @@
         </is>
       </c>
       <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="24" t="inlineStr">
+      <c r="L19" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21748,7 +21454,7 @@
         </is>
       </c>
       <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="24" t="inlineStr">
+      <c r="L20" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21818,7 +21524,7 @@
         </is>
       </c>
       <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="24" t="inlineStr">
+      <c r="L21" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21889,7 +21595,7 @@
         </is>
       </c>
       <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="24" t="inlineStr">
+      <c r="L22" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -21957,7 +21663,7 @@
         </is>
       </c>
       <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="24" t="inlineStr">
+      <c r="L23" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22029,7 +21735,7 @@
         </is>
       </c>
       <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="24" t="inlineStr">
+      <c r="L24" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22099,7 +21805,7 @@
         </is>
       </c>
       <c r="K25" s="28" t="inlineStr"/>
-      <c r="L25" s="24" t="inlineStr">
+      <c r="L25" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22169,7 +21875,7 @@
         </is>
       </c>
       <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="24" t="inlineStr">
+      <c r="L26" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22240,7 +21946,7 @@
         </is>
       </c>
       <c r="K27" s="28" t="inlineStr"/>
-      <c r="L27" s="24" t="inlineStr">
+      <c r="L27" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22311,7 +22017,7 @@
         </is>
       </c>
       <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="24" t="inlineStr">
+      <c r="L28" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22382,7 +22088,7 @@
         </is>
       </c>
       <c r="K29" s="28" t="inlineStr"/>
-      <c r="L29" s="24" t="inlineStr">
+      <c r="L29" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22452,7 +22158,7 @@
         </is>
       </c>
       <c r="K30" s="23" t="inlineStr"/>
-      <c r="L30" s="24" t="inlineStr">
+      <c r="L30" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22522,7 +22228,7 @@
         </is>
       </c>
       <c r="K31" s="28" t="inlineStr"/>
-      <c r="L31" s="24" t="inlineStr">
+      <c r="L31" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22591,7 +22297,7 @@
         </is>
       </c>
       <c r="K32" s="23" t="inlineStr"/>
-      <c r="L32" s="24" t="inlineStr">
+      <c r="L32" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22661,7 +22367,7 @@
         </is>
       </c>
       <c r="K33" s="28" t="inlineStr"/>
-      <c r="L33" s="24" t="inlineStr">
+      <c r="L33" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22731,7 +22437,7 @@
         </is>
       </c>
       <c r="K34" s="23" t="inlineStr"/>
-      <c r="L34" s="24" t="inlineStr">
+      <c r="L34" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22800,7 +22506,7 @@
         </is>
       </c>
       <c r="K35" s="28" t="inlineStr"/>
-      <c r="L35" s="24" t="inlineStr">
+      <c r="L35" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22870,7 +22576,7 @@
         </is>
       </c>
       <c r="K36" s="23" t="inlineStr"/>
-      <c r="L36" s="24" t="inlineStr">
+      <c r="L36" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -22939,7 +22645,7 @@
         </is>
       </c>
       <c r="K37" s="28" t="inlineStr"/>
-      <c r="L37" s="24" t="inlineStr">
+      <c r="L37" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -23008,7 +22714,7 @@
         </is>
       </c>
       <c r="K38" s="23" t="inlineStr"/>
-      <c r="L38" s="24" t="inlineStr">
+      <c r="L38" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -23078,7 +22784,7 @@
         </is>
       </c>
       <c r="K39" s="28" t="inlineStr"/>
-      <c r="L39" s="24" t="inlineStr">
+      <c r="L39" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -23146,7 +22852,7 @@
         </is>
       </c>
       <c r="K40" s="23" t="inlineStr"/>
-      <c r="L40" s="24" t="inlineStr">
+      <c r="L40" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -23216,7 +22922,7 @@
         </is>
       </c>
       <c r="K41" s="28" t="inlineStr"/>
-      <c r="L41" s="24" t="inlineStr">
+      <c r="L41" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>
@@ -23286,7 +22992,7 @@
         </is>
       </c>
       <c r="K42" s="23" t="inlineStr"/>
-      <c r="L42" s="24" t="inlineStr">
+      <c r="L42" s="30" t="inlineStr">
         <is>
           <t>Not Run</t>
         </is>

</xml_diff>

<commit_message>
doc: add folder bug-evidence
</commit_message>
<xml_diff>
--- a/Tests/excel/academic_portal_all_test_cases.xlsx
+++ b/Tests/excel/academic_portal_all_test_cases.xlsx
@@ -1,23 +1,23 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Report" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 01" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 02" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 03" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 04" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 05" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 06" sheetId="8" state="visible" r:id="rId8"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 07" sheetId="9" state="visible" r:id="rId9"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 08" sheetId="10" state="visible" r:id="rId10"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Module 09" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="Report" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="Module 01" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="Module 02" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Module 03" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Module 04" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="Module 05" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="Module 06" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="Module 07" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="Module 08" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="Module 09" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'Module 01'!$A$1:$O$34</definedName>
@@ -497,14 +497,13 @@
 </file>
 
 <file path=xl/charts/chart1.xml><?xml version="1.0" encoding="utf-8"?>
-<chartSpace xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
-  <style val="10"/>
+<chartSpace xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns="http://schemas.openxmlformats.org/drawingml/2006/chart">
   <chart>
     <title>
       <tx>
         <rich>
-          <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-          <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:bodyPr/>
+          <a:p>
             <a:pPr>
               <a:defRPr/>
             </a:pPr>
@@ -528,10 +527,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="FF0000"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -555,10 +554,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="FFFF00"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -582,10 +581,10 @@
             </strRef>
           </tx>
           <spPr>
-            <a:solidFill xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:solidFill>
               <a:srgbClr val="00FF00"/>
             </a:solidFill>
-            <a:ln xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+            <a:ln>
               <a:prstDash val="solid"/>
             </a:ln>
           </spPr>
@@ -614,8 +613,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -641,8 +640,8 @@
         <title>
           <tx>
             <rich>
-              <a:bodyPr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main"/>
-              <a:p xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+              <a:bodyPr/>
+              <a:p>
                 <a:pPr>
                   <a:defRPr/>
                 </a:pPr>
@@ -668,7 +667,7 @@
 </file>
 
 <file path=xl/drawings/drawing1.xml><?xml version="1.0" encoding="utf-8"?>
-<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+<wsDr xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
       <col>6</col>
@@ -683,9 +682,9 @@
         <cNvGraphicFramePr/>
       </nvGraphicFramePr>
       <xfrm/>
-      <a:graphic xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+      <a:graphic>
         <a:graphicData uri="http://schemas.openxmlformats.org/drawingml/2006/chart">
-          <c:chart xmlns:c="http://schemas.openxmlformats.org/drawingml/2006/chart" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+          <c:chart r:id="rId1"/>
         </a:graphicData>
       </a:graphic>
     </graphicFrame>
@@ -20241,10 +20240,15 @@
 New category name "Foundations" is updated and displayed on UI.</t>
         </is>
       </c>
-      <c r="K2" s="23" t="inlineStr"/>
-      <c r="L2" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K2" s="23" t="inlineStr">
+        <is>
+          <t>Category renamed successfully.
+New category name "Foundations" is updated and displayed on UI.</t>
+        </is>
+      </c>
+      <c r="L2" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M2" s="21" t="inlineStr"/>
@@ -20313,10 +20317,15 @@
 Validation error message appears: "Category Name cannot be empty."</t>
         </is>
       </c>
-      <c r="K3" s="28" t="inlineStr"/>
-      <c r="L3" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K3" s="28" t="inlineStr">
+        <is>
+          <t>System blocks action.
+Validation error message appears: "Category Name cannot be empty."</t>
+        </is>
+      </c>
+      <c r="L3" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M3" s="26" t="inlineStr"/>
@@ -20384,10 +20393,14 @@
           <t>Archive and Delete buttons are not present in Category context menu.</t>
         </is>
       </c>
-      <c r="K4" s="23" t="inlineStr"/>
-      <c r="L4" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K4" s="23" t="inlineStr">
+        <is>
+          <t>Archive and Delete buttons are not present in Category context menu.</t>
+        </is>
+      </c>
+      <c r="L4" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M4" s="21" t="inlineStr"/>
@@ -20454,10 +20467,14 @@
           <t>Default categories "IT", "English", and "Professional Skills" are present in system.</t>
         </is>
       </c>
-      <c r="K5" s="28" t="inlineStr"/>
-      <c r="L5" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K5" s="28" t="inlineStr">
+        <is>
+          <t>Default categories "IT", "English", and "Professional Skills" are present in system.</t>
+        </is>
+      </c>
+      <c r="L5" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M5" s="26" t="inlineStr"/>
@@ -20528,10 +20545,15 @@
 New course "Web Development" appears under category "IT".</t>
         </is>
       </c>
-      <c r="K6" s="23" t="inlineStr"/>
-      <c r="L6" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K6" s="23" t="inlineStr">
+        <is>
+          <t>Course created successfully.
+New course "Web Development" appears under category "IT".</t>
+        </is>
+      </c>
+      <c r="L6" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M6" s="21" t="inlineStr"/>
@@ -20599,10 +20621,15 @@
 Validation error appears: "Course Name is required."</t>
         </is>
       </c>
-      <c r="K7" s="28" t="inlineStr"/>
-      <c r="L7" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K7" s="28" t="inlineStr">
+        <is>
+          <t>System blocks action.
+Validation error appears: "Course Name is required."</t>
+        </is>
+      </c>
+      <c r="L7" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M7" s="26" t="inlineStr"/>
@@ -20672,10 +20699,14 @@
           <t>Course name updated successfully to "Frontend Development".</t>
         </is>
       </c>
-      <c r="K8" s="23" t="inlineStr"/>
-      <c r="L8" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K8" s="23" t="inlineStr">
+        <is>
+          <t>Course name updated successfully to "Frontend Development".</t>
+        </is>
+      </c>
+      <c r="L8" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M8" s="21" t="inlineStr"/>
@@ -20744,10 +20775,15 @@
 Course is hidden from Active list and moved to Archived tab.</t>
         </is>
       </c>
-      <c r="K9" s="28" t="inlineStr"/>
-      <c r="L9" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K9" s="28" t="inlineStr">
+        <is>
+          <t>Course status changes to Archived.
+Course is hidden from Active list and moved to Archived tab.</t>
+        </is>
+      </c>
+      <c r="L9" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M9" s="26" t="inlineStr"/>
@@ -20817,10 +20853,15 @@
 Course reappears in active course list.</t>
         </is>
       </c>
-      <c r="K10" s="23" t="inlineStr"/>
-      <c r="L10" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K10" s="23" t="inlineStr">
+        <is>
+          <t>Course status changes back to Active.
+Course reappears in active course list.</t>
+        </is>
+      </c>
+      <c r="L10" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M10" s="21" t="inlineStr"/>
@@ -20888,10 +20929,14 @@
           <t>Permanent Delete button is not present for courses (only Archive is supported).</t>
         </is>
       </c>
-      <c r="K11" s="28" t="inlineStr"/>
-      <c r="L11" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K11" s="28" t="inlineStr">
+        <is>
+          <t>Permanent Delete button is not present for courses (only Archive is supported).</t>
+        </is>
+      </c>
+      <c r="L11" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M11" s="26" t="inlineStr"/>
@@ -20962,10 +21007,15 @@
 "Session 1: HTML Basics" appears inside course.</t>
         </is>
       </c>
-      <c r="K12" s="23" t="inlineStr"/>
-      <c r="L12" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K12" s="23" t="inlineStr">
+        <is>
+          <t>Session created successfully.
+"Session 1: HTML Basics" appears inside course.</t>
+        </is>
+      </c>
+      <c r="L12" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M12" s="21" t="inlineStr"/>
@@ -21033,10 +21083,15 @@
 Validation error appears: "Session Name is required."</t>
         </is>
       </c>
-      <c r="K13" s="28" t="inlineStr"/>
-      <c r="L13" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K13" s="28" t="inlineStr">
+        <is>
+          <t>System blocks action.
+Validation error appears: "Session Name is required."</t>
+        </is>
+      </c>
+      <c r="L13" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M13" s="26" t="inlineStr"/>
@@ -21105,10 +21160,14 @@
           <t>Session details updated successfully.</t>
         </is>
       </c>
-      <c r="K14" s="23" t="inlineStr"/>
-      <c r="L14" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K14" s="23" t="inlineStr">
+        <is>
+          <t>Session details updated successfully.</t>
+        </is>
+      </c>
+      <c r="L14" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M14" s="21" t="inlineStr"/>
@@ -21176,10 +21235,14 @@
           <t>Session and all attached materials are permanently deleted from system.</t>
         </is>
       </c>
-      <c r="K15" s="28" t="inlineStr"/>
-      <c r="L15" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K15" s="28" t="inlineStr">
+        <is>
+          <t>Session and all attached materials are permanently deleted from system.</t>
+        </is>
+      </c>
+      <c r="L15" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M15" s="26" t="inlineStr"/>
@@ -21248,10 +21311,15 @@
 Session remains intact in course.</t>
         </is>
       </c>
-      <c r="K16" s="23" t="inlineStr"/>
-      <c r="L16" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K16" s="23" t="inlineStr">
+        <is>
+          <t>Dialog closes.
+Session remains intact in course.</t>
+        </is>
+      </c>
+      <c r="L16" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M16" s="21" t="inlineStr"/>
@@ -21317,10 +21385,14 @@
           <t>Archive button is not available for sessions (only Delete is supported).</t>
         </is>
       </c>
-      <c r="K17" s="28" t="inlineStr"/>
-      <c r="L17" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K17" s="28" t="inlineStr">
+        <is>
+          <t>Archive button is not available for sessions (only Delete is supported).</t>
+        </is>
+      </c>
+      <c r="L17" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M17" s="26" t="inlineStr"/>
@@ -21391,10 +21463,15 @@
 "Midterm Exam" displays in exam section of course.</t>
         </is>
       </c>
-      <c r="K18" s="23" t="inlineStr"/>
-      <c r="L18" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K18" s="23" t="inlineStr">
+        <is>
+          <t>Exam created successfully.
+"Midterm Exam" displays in exam section of course.</t>
+        </is>
+      </c>
+      <c r="L18" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M18" s="21" t="inlineStr"/>
@@ -21462,10 +21539,15 @@
 Validation error appears: "Exam Name is required."</t>
         </is>
       </c>
-      <c r="K19" s="28" t="inlineStr"/>
-      <c r="L19" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K19" s="28" t="inlineStr">
+        <is>
+          <t>System blocks action.
+Validation error appears: "Exam Name is required."</t>
+        </is>
+      </c>
+      <c r="L19" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M19" s="26" t="inlineStr"/>
@@ -21534,10 +21616,14 @@
           <t>Exam details updated successfully.</t>
         </is>
       </c>
-      <c r="K20" s="23" t="inlineStr"/>
-      <c r="L20" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K20" s="23" t="inlineStr">
+        <is>
+          <t>Exam details updated successfully.</t>
+        </is>
+      </c>
+      <c r="L20" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M20" s="21" t="inlineStr"/>
@@ -21605,10 +21691,14 @@
           <t>Exam and all attached exam materials are permanently deleted from system.</t>
         </is>
       </c>
-      <c r="K21" s="28" t="inlineStr"/>
-      <c r="L21" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K21" s="28" t="inlineStr">
+        <is>
+          <t>Exam and all attached exam materials are permanently deleted from system.</t>
+        </is>
+      </c>
+      <c r="L21" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M21" s="26" t="inlineStr"/>
@@ -21677,10 +21767,15 @@
 Exam remains intact in course.</t>
         </is>
       </c>
-      <c r="K22" s="23" t="inlineStr"/>
-      <c r="L22" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K22" s="23" t="inlineStr">
+        <is>
+          <t>Dialog closes.
+Exam remains intact in course.</t>
+        </is>
+      </c>
+      <c r="L22" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M22" s="21" t="inlineStr"/>
@@ -21746,10 +21841,14 @@
           <t>Archive button is not available for exams (only Delete is supported).</t>
         </is>
       </c>
-      <c r="K23" s="28" t="inlineStr"/>
-      <c r="L23" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K23" s="28" t="inlineStr">
+        <is>
+          <t>Archive button is not available for exams (only Delete is supported).</t>
+        </is>
+      </c>
+      <c r="L23" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M23" s="26" t="inlineStr"/>
@@ -21819,10 +21918,14 @@
           <t>Material link is attached successfully and clickable on UI.</t>
         </is>
       </c>
-      <c r="K24" s="23" t="inlineStr"/>
-      <c r="L24" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K24" s="23" t="inlineStr">
+        <is>
+          <t>Material link is attached successfully and clickable on UI.</t>
+        </is>
+      </c>
+      <c r="L24" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M24" s="21" t="inlineStr"/>
@@ -21890,10 +21993,14 @@
           <t>All material links are attached and displayed under session/exam.</t>
         </is>
       </c>
-      <c r="K25" s="28" t="inlineStr"/>
-      <c r="L25" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K25" s="28" t="inlineStr">
+        <is>
+          <t>All material links are attached and displayed under session/exam.</t>
+        </is>
+      </c>
+      <c r="L25" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M25" s="26" t="inlineStr"/>
@@ -21961,10 +22068,14 @@
           <t>System saves Row 1 successfully and ignores blank Row 2 without error.</t>
         </is>
       </c>
-      <c r="K26" s="23" t="inlineStr"/>
-      <c r="L26" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K26" s="23" t="inlineStr">
+        <is>
+          <t>System saves Row 1 successfully and ignores blank Row 2 without error.</t>
+        </is>
+      </c>
+      <c r="L26" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M26" s="21" t="inlineStr"/>
@@ -22033,13 +22144,17 @@
 Validation error appears: "URL is required when Label is specified."</t>
         </is>
       </c>
-      <c r="K27" s="28" t="inlineStr"/>
-      <c r="L27" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M27" s="26" t="inlineStr"/>
+      <c r="K27" s="28" t="inlineStr">
+        <is>
+          <t>The system saves the document link successfully even though the URL field is empty. No validation error message is displayed, and the attached document link does not appear in the document list after saving.</t>
+        </is>
+      </c>
+      <c r="L27" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="M27" s="26" t="n"/>
       <c r="N27" s="25" t="inlineStr">
         <is>
           <t>High</t>
@@ -22105,13 +22220,17 @@
 Validation error appears: "Label is required when URL is specified."</t>
         </is>
       </c>
-      <c r="K28" s="23" t="inlineStr"/>
-      <c r="L28" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M28" s="21" t="inlineStr"/>
+      <c r="K28" s="23" t="inlineStr">
+        <is>
+          <t>The system saves the document link successfully even though the Label field is empty. No validation error message is displayed, and the attached document link does not appear in the document list after saving.</t>
+        </is>
+      </c>
+      <c r="L28" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="M28" s="21" t="n"/>
       <c r="N28" s="25" t="inlineStr">
         <is>
           <t>High</t>
@@ -22177,10 +22296,15 @@
 Validation error appears: "Material link must be a valid Google Drive URL."</t>
         </is>
       </c>
-      <c r="K29" s="28" t="inlineStr"/>
-      <c r="L29" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K29" s="28" t="inlineStr">
+        <is>
+          <t>System blocks action.
+Validation error appears: "Material link must be a valid Google Drive URL."</t>
+        </is>
+      </c>
+      <c r="L29" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M29" s="26" t="inlineStr"/>
@@ -22248,10 +22372,14 @@
           <t>CSV file downloads successfully containing Session ID, Session Name, and Material details.</t>
         </is>
       </c>
-      <c r="K30" s="23" t="inlineStr"/>
-      <c r="L30" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K30" s="23" t="inlineStr">
+        <is>
+          <t>CSV file downloads successfully containing Session ID, Session Name, and Material details.</t>
+        </is>
+      </c>
+      <c r="L30" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M30" s="21" t="inlineStr"/>
@@ -22319,10 +22447,14 @@
           <t>Session SES-001 is updated with new name "Updated HTML Basics".</t>
         </is>
       </c>
-      <c r="K31" s="28" t="inlineStr"/>
-      <c r="L31" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K31" s="28" t="inlineStr">
+        <is>
+          <t>Session SES-001 is updated with new name "Updated HTML Basics".</t>
+        </is>
+      </c>
+      <c r="L31" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M31" s="26" t="inlineStr"/>
@@ -22389,10 +22521,14 @@
           <t>New session "New CSS Grid Session" is created with auto-generated Session ID.</t>
         </is>
       </c>
-      <c r="K32" s="23" t="inlineStr"/>
-      <c r="L32" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K32" s="23" t="inlineStr">
+        <is>
+          <t>New session "New CSS Grid Session" is created with auto-generated Session ID.</t>
+        </is>
+      </c>
+      <c r="L32" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M32" s="21" t="inlineStr"/>
@@ -22460,13 +22596,19 @@
           <t>New session "Flexbox Guide" is created in system.</t>
         </is>
       </c>
-      <c r="K33" s="28" t="inlineStr"/>
-      <c r="L33" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
-        </is>
-      </c>
-      <c r="M33" s="26" t="inlineStr"/>
+      <c r="K33" s="28" t="inlineStr">
+        <is>
+          <t>The system does not create a new session when importing a row with a non-existing Session ID. Instead, the row is skipped and the message "Row 2: session ID 3 not found." is displayed. No changes are made to the existing sessions.</t>
+        </is>
+      </c>
+      <c r="L33" s="25" t="inlineStr">
+        <is>
+          <t>Failed</t>
+        </is>
+      </c>
+      <c r="M33" s="26" t="e">
+        <v>#VALUE!</v>
+      </c>
       <c r="N33" s="29" t="inlineStr">
         <is>
           <t>Medium</t>
@@ -22531,10 +22673,14 @@
           <t>SES-001 is processed, and omitted session SES-002 remains unchanged in system without being deleted.</t>
         </is>
       </c>
-      <c r="K34" s="23" t="inlineStr"/>
-      <c r="L34" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K34" s="23" t="inlineStr">
+        <is>
+          <t>SES-001 is processed, and omitted session SES-002 remains unchanged in system without being deleted.</t>
+        </is>
+      </c>
+      <c r="L34" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M34" s="21" t="inlineStr"/>
@@ -22601,10 +22747,14 @@
           <t>Sessions are updated/created, and Materials column is safely ignored per business rule.</t>
         </is>
       </c>
-      <c r="K35" s="28" t="inlineStr"/>
-      <c r="L35" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K35" s="28" t="inlineStr">
+        <is>
+          <t>Sessions are updated/created, and Materials column is safely ignored per business rule.</t>
+        </is>
+      </c>
+      <c r="L35" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M35" s="26" t="inlineStr"/>
@@ -22672,10 +22822,15 @@
 Error message appears: "Invalid file format. Please upload a CSV file."</t>
         </is>
       </c>
-      <c r="K36" s="23" t="inlineStr"/>
-      <c r="L36" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K36" s="23" t="inlineStr">
+        <is>
+          <t>System blocks import.
+Error message appears: "Invalid file format. Please upload a CSV file."</t>
+        </is>
+      </c>
+      <c r="L36" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M36" s="21" t="inlineStr"/>
@@ -22742,10 +22897,14 @@
           <t>System flags error for row or skips invalid row with warning message: "Session Name is required."</t>
         </is>
       </c>
-      <c r="K37" s="28" t="inlineStr"/>
-      <c r="L37" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K37" s="28" t="inlineStr">
+        <is>
+          <t>System flags error for row or skips invalid row with warning message: "Session Name is required."</t>
+        </is>
+      </c>
+      <c r="L37" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M37" s="26" t="inlineStr"/>
@@ -22812,10 +22971,14 @@
           <t>Staff user can perform all management operations cleanly.</t>
         </is>
       </c>
-      <c r="K38" s="23" t="inlineStr"/>
-      <c r="L38" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K38" s="23" t="inlineStr">
+        <is>
+          <t>Staff user can perform all management operations cleanly.</t>
+        </is>
+      </c>
+      <c r="L38" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M38" s="21" t="inlineStr"/>
@@ -22883,10 +23046,15 @@
 Student can view and open material links in Read-Only mode.</t>
         </is>
       </c>
-      <c r="K39" s="28" t="inlineStr"/>
-      <c r="L39" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K39" s="28" t="inlineStr">
+        <is>
+          <t>Create, Edit, Archive, Delete, and CSV Import buttons are completely hidden.
+Student can view and open material links in Read-Only mode.</t>
+        </is>
+      </c>
+      <c r="L39" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M39" s="26" t="inlineStr"/>
@@ -22952,10 +23120,14 @@
           <t>Access denied page or login redirect is displayed.</t>
         </is>
       </c>
-      <c r="K40" s="23" t="inlineStr"/>
-      <c r="L40" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K40" s="23" t="inlineStr">
+        <is>
+          <t>Access denied page or login redirect is displayed.</t>
+        </is>
+      </c>
+      <c r="L40" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M40" s="21" t="inlineStr"/>
@@ -23023,10 +23195,14 @@
           <t>Course and all its child sessions and exams are hidden from active view.</t>
         </is>
       </c>
-      <c r="K41" s="28" t="inlineStr"/>
-      <c r="L41" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K41" s="28" t="inlineStr">
+        <is>
+          <t>Course and all its child sessions and exams are hidden from active view.</t>
+        </is>
+      </c>
+      <c r="L41" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M41" s="26" t="inlineStr"/>
@@ -23094,10 +23270,14 @@
           <t>Course and all child sessions and exams reappear in active view.</t>
         </is>
       </c>
-      <c r="K42" s="23" t="inlineStr"/>
-      <c r="L42" s="30" t="inlineStr">
-        <is>
-          <t>Not Run</t>
+      <c r="K42" s="23" t="inlineStr">
+        <is>
+          <t>Course and all child sessions and exams reappear in active view.</t>
+        </is>
+      </c>
+      <c r="L42" s="24" t="inlineStr">
+        <is>
+          <t>Passed</t>
         </is>
       </c>
       <c r="M42" s="21" t="inlineStr"/>

</xml_diff>